<commit_message>
New electronics links in BOM
</commit_message>
<xml_diff>
--- a/P01/P01_06_Procurement/Table_260719_BOM.xlsx
+++ b/P01/P01_06_Procurement/Table_260719_BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A1097411\Documents\GitHub\ORGOfly-CAD-Model\P01\P01_06_Procurement\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\ORGOfly\ORGOfly-CAD-model\P01\P01_06_Procurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF97DF5-F8CA-47A0-BB99-1F65A6C25E92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DAC9899-B003-4074-BB18-71E93D38844D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{EEE73C29-3BDB-49EB-9C57-2FAD514C20AA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{EEE73C29-3BDB-49EB-9C57-2FAD514C20AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Background_info" sheetId="2" state="hidden" r:id="rId1"/>
@@ -37,8 +37,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="146">
   <si>
     <t>#</t>
   </si>
@@ -262,21 +284,9 @@
     <t>https://hobbyking.com/en_us/turnigy-heavy-duty-5500mah-6s-60c-lipo-pack-w-xt90.html</t>
   </si>
   <si>
-    <t>https://n-factory.de/F405-WING_15?srsltid=AfmBOorJLigbjhDd51Re4u0jHc0Jw6epVL2ePDy3WgvZ8yOpSwySAvJh</t>
-  </si>
-  <si>
     <t>Sold in bulk</t>
   </si>
   <si>
-    <t>https://sequremall.com/products/sequre-12100-brushless-electric-speed-controller-5-12s-power-supply-100a-blheli_32-am32-firmware-support-128khz-pwm-frequency-suitable-for-multi-rotor-aircrafts-airplane-models-plant-protection-machine-boat-models-rc-car-models?srsltid=AfmBOoqD3cKLbLKnMnpXxBff0019A01XQKeqCUJ8P-pC8NoTSW-f13nF</t>
-  </si>
-  <si>
-    <t>Sold in bulk. 8 pairs needed</t>
-  </si>
-  <si>
-    <t>https://www.amazon.de/-/en/HAXIHA-Battery-Connectors-Connector-Current-Pack-20-XT90/dp/B0F8914WTT/ref=sr_1_8?crid=3OZBHNPL6RRCJ&amp;dib=eyJ2IjoiMSJ9.ELU5HE2AqFpDy8xZeyhowEBvzt0Jdvcoxheaz9pNyfWQqI8F7CHyE9iCFhhg2h1SfLmhIaMf1mNFh9H62Nxwja70hUmdhOfmhzY2CjDv70npxhA_c3MXC-zkVkeBttQdMU1Zdq9_KBYeElfuxRMIk5K7A0gtovw9QVCSFDZ4dFhSAdp7nSFB3va-wbwVjV_zQ0HR6w-aVbGPjeNxzewu9FPPXFicV7UguDyyznJctKq4LMokyDPwK2vE1ICdVmh2oS_o5aBV0FPE3K90fGSupxQWjFk76sR791TqqYw8G0s.s4r_dP4cebl1DPDP7JN6xQxZe1hPSZwhB17M5TXeC-o&amp;dib_tag=se&amp;keywords=xt90%2Bstecker&amp;qid=1781937738&amp;sprefix=xt90%2Caps%2C438&amp;sr=8-8&amp;th=1</t>
-  </si>
-  <si>
     <t>Pack of 20 XT90 Battery Connectors (10 pairs)</t>
   </si>
   <si>
@@ -328,19 +338,7 @@
     <t>Sold in bulk. 4 500KV motors</t>
   </si>
   <si>
-    <t>https://www.drone-fpv-racer.com/en/pdb-fchub-12s-v2-440a-bec-512v-by-matek-10435.html</t>
-  </si>
-  <si>
     <t>4-10 days</t>
-  </si>
-  <si>
-    <t>https://n-factory.de/TBS-Crossfire-Diversity-Nano-RX-Receiver-FPV-Long-Range_1</t>
-  </si>
-  <si>
-    <t>Order from the same place as FC and PDB for cheaper delivery</t>
-  </si>
-  <si>
-    <t>Order from the same place as FC and RX for cheaper delivery</t>
   </si>
   <si>
     <t>Order from the same place as RX and PDB for cheaper delivery</t>
@@ -456,14 +454,62 @@
     <t>D-Shafts would be manually manufactured using 5mm aluminum rods</t>
   </si>
   <si>
-    <t>Total Spent</t>
+    <t>No EU Availability</t>
+  </si>
+  <si>
+    <t>Core propulsion system component</t>
+  </si>
+  <si>
+    <t>Ovonic Roam 6S 5Ah5 150C  XT90-S</t>
+  </si>
+  <si>
+    <t>5-9 days</t>
+  </si>
+  <si>
+    <t>https://www.ampow.com/products/ovonic-roam-series-6s-lipo-battery-5500mah-6s1p-150c-22-2v-long-range-lipo-battery-with-xt90-s-anti-spark-plug-for-6s-cinelifte-drone-multirotor-x-class?_pos=39&amp;_fid=ed406fb17&amp;_ss=c</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005006753480927.html?gatewayAdapt=deu2glo</t>
+  </si>
+  <si>
+    <t>Can also be bought for 49.99USD with 12USD shipping from sequermall.com</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005012792435664.html</t>
+  </si>
+  <si>
+    <t>10-20 days</t>
+  </si>
+  <si>
+    <t>Sold in bulk. 8 pairs needed. Can also be ordered of amazon https://www.amazon.de/-/en/HAXIHA-Battery-Connectors-Connector-Current-Pack-20-XT90/dp/B0F8914WTT/ref=sr_1_8?crid=3OZBHNPL6RRCJ&amp;dib=eyJ2IjoiMSJ9.ELU5HE2AqFpDy8xZeyhowEBvzt0Jdvcoxheaz9pNyfWQqI8F7CHyE9iCFhhg2h1SfLmhIaMf1mNFh9H62Nxwja70hUmdhOfmhzY2CjDv70npxhA_c3MXC-zkVkeBttQdMU1Zdq9_KBYeElfuxRMIk5K7A0gtovw9QVCSFDZ4dFhSAdp7nSFB3va-wbwVjV_zQ0HR6w-aVbGPjeNxzewu9FPPXFicV7UguDyyznJctKq4LMokyDPwK2vE1ICdVmh2oS_o5aBV0FPE3K90fGSupxQWjFk76sR791TqqYw8G0s.s4r_dP4cebl1DPDP7JN6xQxZe1hPSZwhB17M5TXeC-o&amp;dib_tag=se&amp;keywords=xt90%2Bstecker&amp;qid=1781937738&amp;sprefix=xt90%2Caps%2C438&amp;sr=8-8&amp;th=1</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005003122596249.html?spm=a2g0o.productlist.main.23.70394477bJf9UQ&amp;algo_pvid=169d2b7f-426b-4582-b7f2-1a69c234abe7&amp;algo_exp_id=169d2b7f-426b-4582-b7f2-1a69c234abe7-20&amp;pdp_ext_f=%7B%22order%22%3A%222145%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%217.69%215.92%21%21%218.62%216.64%21%400b8848e317897611280765333e0f49%2112000024217621966%21sea%21BG%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3Abb4150ed%3Bm03_new_user%3A-29895%3BpisId%3A5000000217831009&amp;curPageLogUid=7PGL6jiPmM9H&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005003122596249%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>3-5 days</t>
+  </si>
+  <si>
+    <t>https://www.rotorama.de/product/matek-xclass-pdb-fchub-12s</t>
+  </si>
+  <si>
+    <t>Delivery with ECONT. Cheaper delivery options available</t>
+  </si>
+  <si>
+    <t>https://n-factory.de/TBS-Crossfire-Diversity-Nano-RX-Receiver-FPV-Long-Range_1?srsltid=AU7gw4Vx0tsp-ivZWozvmeD9z-vS4TeDNtS8Ba--6kkVj-S0ciJFwk-R</t>
+  </si>
+  <si>
+    <t>Available (fow now). We need to contact them separately for ordering</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9" x14ac:knownFonts="1">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -534,8 +580,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -557,6 +609,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -615,7 +679,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -656,7 +720,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -701,12 +764,24 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1086,12 +1161,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B02F099F-610B-4C2F-A80F-3888BDD56E8E}">
   <dimension ref="B2:D14"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="4" max="4" width="33.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:4" ht="15">
       <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
@@ -1102,7 +1177,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4">
       <c r="B3" t="s">
         <v>4</v>
       </c>
@@ -1113,7 +1188,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:4">
       <c r="B4" t="s">
         <v>6</v>
       </c>
@@ -1124,7 +1199,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:4">
       <c r="B5" t="s">
         <v>5</v>
       </c>
@@ -1135,7 +1210,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:4">
       <c r="B6" t="s">
         <v>7</v>
       </c>
@@ -1146,9 +1221,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:4">
       <c r="B7" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="C7" t="s">
         <v>13</v>
@@ -1157,37 +1232,37 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:4">
       <c r="D8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:4">
       <c r="D9" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:4">
       <c r="D10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:4">
       <c r="D11" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:4">
       <c r="D12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:4">
       <c r="D13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:4">
       <c r="D14" t="s">
         <v>21</v>
       </c>
@@ -1199,33 +1274,33 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E734346-BCBC-4D9C-B399-F93315446069}">
-  <dimension ref="A1:N38"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:N39"/>
+  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="3" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="30.44140625" style="7" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="30.5" style="7" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" style="2" customWidth="1"/>
-    <col min="4" max="4" width="37.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="8.88671875" style="1"/>
-    <col min="7" max="7" width="8.21875" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.33203125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.88671875" style="1"/>
+    <col min="4" max="4" width="37.625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="8.875" style="1"/>
+    <col min="7" max="7" width="8.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.375" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.375" style="1" customWidth="1"/>
+    <col min="11" max="11" width="9.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.875" style="1"/>
     <col min="13" max="13" width="55" style="17" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="60.77734375" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.88671875" style="2"/>
+    <col min="14" max="14" width="60.75" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" ht="15">
       <c r="A1" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C1" s="6"/>
       <c r="M1" s="2"/>
     </row>
-    <row r="2" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" ht="27" customHeight="1">
       <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
@@ -1266,10 +1341,10 @@
         <v>14</v>
       </c>
       <c r="N2" s="11" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
       <c r="A3" s="15">
         <f>IF(B3&lt;&gt;"",COUNTA($B$3:B3),"")</f>
         <v>1</v>
@@ -1301,18 +1376,18 @@
       <c r="K3" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="L3" s="24" t="s">
+      <c r="L3" s="23" t="s">
         <v>36</v>
       </c>
       <c r="M3" s="16"/>
       <c r="N3" s="16"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14">
       <c r="A4" s="15">
         <f>IF(B4&lt;&gt;"",COUNTA($B$3:B4),"")</f>
         <v>2</v>
       </c>
-      <c r="B4" s="27" t="s">
+      <c r="B4" s="26" t="s">
         <v>38</v>
       </c>
       <c r="C4" s="13" t="s">
@@ -1343,7 +1418,7 @@
       <c r="K4" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="L4" s="24" t="s">
+      <c r="L4" s="23" t="s">
         <v>36</v>
       </c>
       <c r="M4" s="16" t="s">
@@ -1351,16 +1426,16 @@
       </c>
       <c r="N4" s="16"/>
     </row>
-    <row r="5" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" ht="28.5">
       <c r="A5" s="15">
         <f>IF(B5&lt;&gt;"",COUNTA($B$3:B5),"")</f>
         <v>3</v>
       </c>
-      <c r="B5" s="27" t="s">
-        <v>121</v>
+      <c r="B5" s="26" t="s">
+        <v>113</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>24</v>
@@ -1375,36 +1450,36 @@
         <v>1</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
       <c r="J5" s="15">
         <f>(G5*E5)+F5</f>
         <v>17.96</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>126</v>
-      </c>
-      <c r="L5" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="L5" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="M5" s="19" t="s">
-        <v>122</v>
+      <c r="M5" s="18" t="s">
+        <v>114</v>
       </c>
       <c r="N5" s="16"/>
     </row>
-    <row r="6" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" ht="42.75">
       <c r="A6" s="15">
         <f>IF(B6&lt;&gt;"",COUNTA($B$3:B6),"")</f>
         <v>4</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="B6" s="26" t="s">
         <v>40</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>24</v>
@@ -1419,32 +1494,32 @@
         <v>1</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="J6" s="15">
         <f>(G6*E6)+F6</f>
         <v>33.32</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>129</v>
-      </c>
-      <c r="L6" s="24" t="s">
+        <v>121</v>
+      </c>
+      <c r="L6" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="M6" s="19" t="s">
-        <v>130</v>
+      <c r="M6" s="18" t="s">
+        <v>122</v>
       </c>
       <c r="N6" s="16"/>
     </row>
-    <row r="7" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" ht="28.5">
       <c r="A7" s="15">
         <f>IF(B7&lt;&gt;"",COUNTA($B$3:B7),"")</f>
         <v>5</v>
       </c>
-      <c r="B7" s="27" t="s">
+      <c r="B7" s="26" t="s">
         <v>37</v>
       </c>
       <c r="C7" s="13" t="s">
@@ -1456,7 +1531,7 @@
       <c r="E7" s="15">
         <v>31.22</v>
       </c>
-      <c r="F7" s="33">
+      <c r="F7" s="32">
         <v>18.75</v>
       </c>
       <c r="G7" s="15">
@@ -1466,29 +1541,29 @@
         <v>4</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="J7" s="15">
-        <f t="shared" ref="J7:J21" si="0">(G7*E7)+F7</f>
+        <f t="shared" ref="J7:J22" si="0">(G7*E7)+F7</f>
         <v>143.63</v>
       </c>
-      <c r="K7" s="25" t="s">
-        <v>134</v>
-      </c>
-      <c r="L7" s="24" t="s">
+      <c r="K7" s="24" t="s">
+        <v>126</v>
+      </c>
+      <c r="L7" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="M7" s="19" t="s">
-        <v>127</v>
+      <c r="M7" s="18" t="s">
+        <v>119</v>
       </c>
       <c r="N7" s="16"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14">
       <c r="A8" s="15">
         <f>IF(B8&lt;&gt;"",COUNTA($B$3:B8),"")</f>
         <v>6</v>
       </c>
-      <c r="B8" s="27" t="s">
+      <c r="B8" s="26" t="s">
         <v>39</v>
       </c>
       <c r="C8" s="13" t="s">
@@ -1500,7 +1575,7 @@
       <c r="E8" s="15">
         <v>12.83</v>
       </c>
-      <c r="F8" s="34"/>
+      <c r="F8" s="33"/>
       <c r="G8" s="15">
         <v>2</v>
       </c>
@@ -1508,29 +1583,29 @@
         <v>4</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>133</v>
+        <v>125</v>
       </c>
       <c r="J8" s="15">
         <f t="shared" si="0"/>
         <v>25.66</v>
       </c>
-      <c r="K8" s="25" t="s">
-        <v>134</v>
-      </c>
-      <c r="L8" s="24" t="s">
+      <c r="K8" s="24" t="s">
+        <v>126</v>
+      </c>
+      <c r="L8" s="23" t="s">
         <v>10</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
       <c r="N8" s="16"/>
     </row>
-    <row r="9" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" ht="28.5">
       <c r="A9" s="15">
         <f>IF(B9&lt;&gt;"",COUNTA($B$3:B9),"")</f>
         <v>7</v>
       </c>
-      <c r="B9" s="27" t="s">
+      <c r="B9" s="26" t="s">
         <v>47</v>
       </c>
       <c r="C9" s="13" t="s">
@@ -1552,7 +1627,7 @@
         <v>4</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
       <c r="J9" s="15">
         <f t="shared" si="0"/>
@@ -1561,20 +1636,20 @@
       <c r="K9" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="L9" s="24" t="s">
+      <c r="L9" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="M9" s="19" t="s">
-        <v>119</v>
-      </c>
-      <c r="N9" s="32"/>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="M9" s="18" t="s">
+        <v>111</v>
+      </c>
+      <c r="N9" s="31"/>
+    </row>
+    <row r="10" spans="1:14" ht="15">
       <c r="A10" s="15">
         <f>IF(B10&lt;&gt;"",COUNTA($B$3:B10),"")</f>
         <v>8</v>
       </c>
-      <c r="B10" s="28" t="s">
+      <c r="B10" s="27" t="s">
         <v>50</v>
       </c>
       <c r="C10" s="13" t="s">
@@ -1596,19 +1671,18 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="K10" s="15"/>
-      <c r="L10" s="24" t="s">
+      <c r="L10" s="23" t="s">
         <v>36</v>
       </c>
       <c r="M10" s="16"/>
       <c r="N10" s="16"/>
     </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14">
       <c r="A11" s="15">
         <f>IF(B11&lt;&gt;"",COUNTA($B$3:B11),"")</f>
         <v>9</v>
       </c>
-      <c r="B11" s="29" t="s">
+      <c r="B11" s="34" t="s">
         <v>57</v>
       </c>
       <c r="C11" s="13" t="s">
@@ -1637,33 +1711,37 @@
         <v>243</v>
       </c>
       <c r="K11" s="15" t="s">
-        <v>107</v>
-      </c>
-      <c r="L11" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="M11" s="16"/>
-      <c r="N11" s="16"/>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+        <v>99</v>
+      </c>
+      <c r="L11" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="M11" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="N11" s="16" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
       <c r="A12" s="15">
-        <f>IF(B12&lt;&gt;"",COUNTA($B$3:B12),"")</f>
-        <v>10</v>
-      </c>
-      <c r="B12" s="27" t="s">
-        <v>105</v>
+        <f>IF(B13&lt;&gt;"",COUNTA($B$3:B13),"")</f>
+        <v>11</v>
+      </c>
+      <c r="B12" s="28" t="s">
+        <v>131</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>103</v>
+        <v>51</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E12" s="15">
-        <v>16.45</v>
+        <v>62.75</v>
       </c>
       <c r="F12" s="15">
-        <v>0</v>
+        <v>24.57</v>
       </c>
       <c r="G12" s="15">
         <v>2</v>
@@ -1671,71 +1749,81 @@
       <c r="H12" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I12" s="3" t="s">
-        <v>104</v>
+      <c r="I12" s="8" t="s">
+        <v>133</v>
       </c>
       <c r="J12" s="15">
         <f t="shared" si="0"/>
-        <v>32.9</v>
-      </c>
-      <c r="K12" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="L12" s="24" t="s">
-        <v>36</v>
+        <v>150.07</v>
+      </c>
+      <c r="K12" s="24" t="s">
+        <v>132</v>
+      </c>
+      <c r="L12" s="23" t="s">
+        <v>10</v>
       </c>
       <c r="M12" s="16" t="s">
-        <v>106</v>
+        <v>130</v>
       </c>
       <c r="N12" s="16"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14">
       <c r="A13" s="15">
-        <f>IF(B13&lt;&gt;"",COUNTA($B$3:B13),"")</f>
-        <v>11</v>
-      </c>
-      <c r="B13" s="29" t="s">
-        <v>56</v>
+        <f>IF(B14&lt;&gt;"",COUNTA($B$3:B14),"")</f>
+        <v>12</v>
+      </c>
+      <c r="B13" s="26" t="s">
+        <v>97</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>52</v>
+        <v>95</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="15"/>
-      <c r="F13" s="15"/>
+        <v>18</v>
+      </c>
+      <c r="E13" s="15">
+        <v>16.45</v>
+      </c>
+      <c r="F13" s="15">
+        <v>0</v>
+      </c>
       <c r="G13" s="15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H13" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I13" s="3"/>
+      <c r="I13" s="3" t="s">
+        <v>96</v>
+      </c>
       <c r="J13" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K13" s="15"/>
-      <c r="L13" s="24" t="s">
+        <v>32.9</v>
+      </c>
+      <c r="K13" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="L13" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="M13" s="16"/>
+      <c r="M13" s="16" t="s">
+        <v>98</v>
+      </c>
       <c r="N13" s="16"/>
     </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14">
       <c r="A14" s="15">
-        <f>IF(B14&lt;&gt;"",COUNTA($B$3:B14),"")</f>
-        <v>12</v>
-      </c>
-      <c r="B14" s="13" t="s">
-        <v>58</v>
+        <f>IF(B15&lt;&gt;"",COUNTA($B$3:B15),"")</f>
+        <v>13</v>
+      </c>
+      <c r="B14" s="34" t="s">
+        <v>56</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E14" s="15"/>
       <c r="F14" s="15"/>
@@ -1751,183 +1839,175 @@
         <v>0</v>
       </c>
       <c r="K14" s="15"/>
-      <c r="L14" s="24" t="s">
+      <c r="L14" s="23" t="s">
         <v>36</v>
       </c>
       <c r="M14" s="16"/>
       <c r="N14" s="16"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14">
       <c r="A15" s="15">
-        <f>IF(B15&lt;&gt;"",COUNTA($B$3:B15),"")</f>
-        <v>13</v>
-      </c>
-      <c r="B15" s="29" t="s">
-        <v>53</v>
+        <f>IF(B16&lt;&gt;"",COUNTA($B$3:B16),"")</f>
+        <v>14</v>
+      </c>
+      <c r="B15" s="13" t="s">
+        <v>58</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E15" s="15">
-        <v>44.99</v>
-      </c>
-      <c r="F15" s="15">
-        <v>19</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
       <c r="G15" s="15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H15" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I15" s="3" t="s">
-        <v>76</v>
-      </c>
+      <c r="I15" s="3"/>
       <c r="J15" s="15">
         <f t="shared" si="0"/>
-        <v>198.96</v>
-      </c>
-      <c r="K15" s="15" t="s">
-        <v>102</v>
-      </c>
-      <c r="L15" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="K15" s="15"/>
+      <c r="L15" s="23" t="s">
         <v>36</v>
       </c>
       <c r="M15" s="16"/>
       <c r="N15" s="16"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14">
       <c r="A16" s="15">
-        <f>IF(B16&lt;&gt;"",COUNTA($B$3:B16),"")</f>
-        <v>14</v>
-      </c>
-      <c r="B16" s="29" t="s">
-        <v>69</v>
+        <f>IF(B17&lt;&gt;"",COUNTA($B$3:B17),"")</f>
+        <v>15</v>
+      </c>
+      <c r="B16" s="28" t="s">
+        <v>53</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="E16" s="15">
-        <v>49.95</v>
+        <v>51.39</v>
       </c>
       <c r="F16" s="15">
-        <v>14.9</v>
+        <v>16.739999999999998</v>
       </c>
       <c r="G16" s="15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I16" s="3" t="s">
-        <v>74</v>
+      <c r="I16" s="8" t="s">
+        <v>134</v>
       </c>
       <c r="J16" s="15">
         <f t="shared" si="0"/>
-        <v>64.850000000000009</v>
+        <v>222.3</v>
       </c>
       <c r="K16" s="15" t="s">
-        <v>97</v>
-      </c>
-      <c r="L16" s="24" t="s">
-        <v>36</v>
+        <v>94</v>
+      </c>
+      <c r="L16" s="23" t="s">
+        <v>10</v>
       </c>
       <c r="M16" s="16" t="s">
-        <v>101</v>
+        <v>135</v>
       </c>
       <c r="N16" s="16"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14">
       <c r="A17" s="15">
-        <f>IF(B17&lt;&gt;"",COUNTA($B$3:B17),"")</f>
-        <v>15</v>
-      </c>
-      <c r="B17" s="27" t="s">
-        <v>54</v>
+        <f>IF(B18&lt;&gt;"",COUNTA($B$3:B18),"")</f>
+        <v>16</v>
+      </c>
+      <c r="B17" s="28" t="s">
+        <v>69</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E17" s="15"/>
-      <c r="F17" s="15"/>
+      <c r="E17" s="15">
+        <v>63.99</v>
+      </c>
+      <c r="F17" s="15">
+        <v>0</v>
+      </c>
       <c r="G17" s="15">
         <v>1</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I17" s="3"/>
+      <c r="I17" s="8" t="s">
+        <v>136</v>
+      </c>
       <c r="J17" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K17" s="15"/>
-      <c r="L17" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="M17" s="16"/>
+        <v>63.99</v>
+      </c>
+      <c r="K17" s="15" t="s">
+        <v>137</v>
+      </c>
+      <c r="L17" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>93</v>
+      </c>
       <c r="N17" s="16"/>
     </row>
-    <row r="18" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14">
       <c r="A18" s="15">
-        <f>IF(B18&lt;&gt;"",COUNTA($B$3:B18),"")</f>
-        <v>16</v>
-      </c>
-      <c r="B18" s="29" t="s">
-        <v>79</v>
+        <f>IF(B19&lt;&gt;"",COUNTA($B$3:B19),"")</f>
+        <v>17</v>
+      </c>
+      <c r="B18" s="26" t="s">
+        <v>54</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>60</v>
+        <v>68</v>
       </c>
       <c r="D18" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="E18" s="15">
-        <v>13.1</v>
-      </c>
-      <c r="F18" s="15">
-        <v>0</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15"/>
       <c r="G18" s="15">
         <v>1</v>
       </c>
       <c r="H18" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I18" s="3" t="s">
-        <v>78</v>
-      </c>
+      <c r="I18" s="3"/>
       <c r="J18" s="15">
         <f t="shared" si="0"/>
-        <v>13.1</v>
-      </c>
-      <c r="K18" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="L18" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="K18" s="15"/>
+      <c r="L18" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="M18" s="16" t="s">
-        <v>77</v>
-      </c>
+      <c r="M18" s="16"/>
       <c r="N18" s="16"/>
     </row>
-    <row r="19" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" ht="28.5">
       <c r="A19" s="15">
-        <f>IF(B19&lt;&gt;"",COUNTA($B$3:B19),"")</f>
-        <v>17</v>
-      </c>
-      <c r="B19" s="27" t="s">
-        <v>81</v>
+        <f>IF(B20&lt;&gt;"",COUNTA($B$3:B20),"")</f>
+        <v>18</v>
+      </c>
+      <c r="B19" s="28" t="s">
+        <v>75</v>
       </c>
       <c r="C19" s="13" t="s">
         <v>60</v>
@@ -1936,51 +2016,51 @@
         <v>30</v>
       </c>
       <c r="E19" s="15">
-        <v>7.04</v>
+        <v>5.92</v>
       </c>
       <c r="F19" s="15">
-        <v>0</v>
+        <v>5.95</v>
       </c>
       <c r="G19" s="15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H19" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I19" s="3" t="s">
-        <v>82</v>
+      <c r="I19" s="8" t="s">
+        <v>139</v>
       </c>
       <c r="J19" s="15">
         <f t="shared" si="0"/>
-        <v>7.04</v>
+        <v>17.79</v>
       </c>
       <c r="K19" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="L19" s="24" t="s">
-        <v>36</v>
+        <v>137</v>
+      </c>
+      <c r="L19" s="23" t="s">
+        <v>10</v>
       </c>
       <c r="M19" s="16" t="s">
-        <v>80</v>
+        <v>138</v>
       </c>
       <c r="N19" s="16"/>
     </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" ht="28.5">
       <c r="A20" s="15">
-        <f>IF(B20&lt;&gt;"",COUNTA($B$3:B20),"")</f>
-        <v>18</v>
-      </c>
-      <c r="B20" s="27" t="s">
-        <v>83</v>
+        <f>IF(B21&lt;&gt;"",COUNTA($B$3:B21),"")</f>
+        <v>19</v>
+      </c>
+      <c r="B20" s="26" t="s">
+        <v>77</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>30</v>
       </c>
       <c r="E20" s="15">
-        <v>14.81</v>
+        <v>7.04</v>
       </c>
       <c r="F20" s="15">
         <v>0</v>
@@ -1992,38 +2072,39 @@
         <v>4</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="J20" s="15">
         <f t="shared" si="0"/>
-        <v>14.81</v>
+        <v>7.04</v>
       </c>
       <c r="K20" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="L20" s="24" t="s">
+      <c r="L20" s="23" t="s">
         <v>36</v>
       </c>
       <c r="M20" s="16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="N20" s="16"/>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14">
       <c r="A21" s="15">
-        <v>19</v>
-      </c>
-      <c r="B21" s="27" t="s">
-        <v>91</v>
+        <f>IF(B22&lt;&gt;"",COUNTA($B$3:B22),"")</f>
+        <v>20</v>
+      </c>
+      <c r="B21" s="26" t="s">
+        <v>79</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>30</v>
       </c>
       <c r="E21" s="15">
-        <v>6.61</v>
+        <v>14.81</v>
       </c>
       <c r="F21" s="15">
         <v>0</v>
@@ -2035,38 +2116,39 @@
         <v>4</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="J21" s="15">
         <f t="shared" si="0"/>
-        <v>6.61</v>
+        <v>14.81</v>
       </c>
       <c r="K21" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="L21" s="24" t="s">
+      <c r="L21" s="23" t="s">
         <v>36</v>
       </c>
       <c r="M21" s="16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="N21" s="16"/>
     </row>
-    <row r="22" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14">
       <c r="A22" s="15">
-        <v>19</v>
-      </c>
-      <c r="B22" s="30" t="s">
+        <f>IF(B23&lt;&gt;"",COUNTA($B$3:B23),"")</f>
+        <v>21</v>
+      </c>
+      <c r="B22" s="26" t="s">
+        <v>87</v>
+      </c>
+      <c r="C22" s="13" t="s">
         <v>85</v>
-      </c>
-      <c r="C22" s="13" t="s">
-        <v>86</v>
       </c>
       <c r="D22" s="15" t="s">
         <v>30</v>
       </c>
       <c r="E22" s="15">
-        <v>8.66</v>
+        <v>6.61</v>
       </c>
       <c r="F22" s="15">
         <v>0</v>
@@ -2077,116 +2159,116 @@
       <c r="H22" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I22" s="13" t="s">
+      <c r="I22" s="3" t="s">
         <v>84</v>
       </c>
       <c r="J22" s="15">
-        <f t="shared" ref="J22:J27" si="1">(G22*E22)+F22</f>
-        <v>8.66</v>
+        <f t="shared" si="0"/>
+        <v>6.61</v>
       </c>
       <c r="K22" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="L22" s="24" t="s">
+      <c r="L22" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="M22" s="16"/>
+      <c r="M22" s="16" t="s">
+        <v>74</v>
+      </c>
       <c r="N22" s="16"/>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" ht="12.75" customHeight="1">
       <c r="A23" s="15">
-        <f>IF(B23&lt;&gt;"",COUNTA($B$3:B23),"")</f>
-        <v>21</v>
-      </c>
-      <c r="B23" s="20" t="s">
-        <v>61</v>
+        <f>IF(B24&lt;&gt;"",COUNTA($B$3:B24),"")</f>
+        <v>22</v>
+      </c>
+      <c r="B23" s="29" t="s">
+        <v>81</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>55</v>
+        <v>82</v>
       </c>
       <c r="D23" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="E23" s="15"/>
-      <c r="F23" s="15"/>
+      <c r="E23" s="15">
+        <v>8.66</v>
+      </c>
+      <c r="F23" s="15">
+        <v>0</v>
+      </c>
       <c r="G23" s="15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H23" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I23" s="3"/>
+      <c r="I23" s="13" t="s">
+        <v>80</v>
+      </c>
       <c r="J23" s="15">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K23" s="15"/>
-      <c r="L23" s="24" t="s">
+        <f t="shared" ref="J23:J28" si="1">(G23*E23)+F23</f>
+        <v>8.66</v>
+      </c>
+      <c r="K23" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="L23" s="23" t="s">
         <v>36</v>
       </c>
       <c r="M23" s="16"/>
       <c r="N23" s="16"/>
     </row>
-    <row r="24" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" ht="15">
       <c r="A24" s="15">
-        <f>IF(B24&lt;&gt;"",COUNTA($B$3:B24),"")</f>
-        <v>22</v>
-      </c>
-      <c r="B24" s="26" t="s">
-        <v>93</v>
+        <f>IF(B25&lt;&gt;"",COUNTA($B$3:B25),"")</f>
+        <v>23</v>
+      </c>
+      <c r="B24" s="19" t="s">
+        <v>61</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="D24" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E24" s="15">
-        <v>170.89</v>
-      </c>
-      <c r="F24" s="15">
-        <v>0</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E24" s="15"/>
+      <c r="F24" s="15"/>
       <c r="G24" s="15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H24" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I24" s="3" t="s">
-        <v>92</v>
-      </c>
+      <c r="I24" s="3"/>
       <c r="J24" s="15">
         <f t="shared" si="1"/>
-        <v>170.89</v>
-      </c>
-      <c r="K24" s="15" t="s">
-        <v>94</v>
-      </c>
-      <c r="L24" s="24" t="s">
+        <v>0</v>
+      </c>
+      <c r="K24" s="15"/>
+      <c r="L24" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="M24" s="16" t="s">
-        <v>95</v>
-      </c>
+      <c r="M24" s="16"/>
       <c r="N24" s="16"/>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" ht="28.5">
       <c r="A25" s="15">
-        <f>IF(B25&lt;&gt;"",COUNTA($B$3:B25),"")</f>
-        <v>23</v>
-      </c>
-      <c r="B25" s="31" t="s">
-        <v>66</v>
+        <f>IF(B26&lt;&gt;"",COUNTA($B$3:B26),"")</f>
+        <v>24</v>
+      </c>
+      <c r="B25" s="25" t="s">
+        <v>89</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E25" s="15">
-        <v>31.9</v>
+        <v>174.99</v>
       </c>
       <c r="F25" s="15">
         <v>0</v>
@@ -2197,41 +2279,43 @@
       <c r="H25" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I25" s="3" t="s">
-        <v>96</v>
+      <c r="I25" s="8" t="s">
+        <v>88</v>
       </c>
       <c r="J25" s="15">
         <f t="shared" si="1"/>
+        <v>174.99</v>
+      </c>
+      <c r="K25" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="L25" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="M25" s="16" t="s">
+        <v>91</v>
+      </c>
+      <c r="N25" s="16"/>
+    </row>
+    <row r="26" spans="1:14">
+      <c r="A26" s="15">
+        <f>IF(B27&lt;&gt;"",COUNTA($B$3:B27),"")</f>
+        <v>25</v>
+      </c>
+      <c r="B26" s="30" t="s">
+        <v>66</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E26" s="15">
         <v>31.9</v>
       </c>
-      <c r="K25" s="15"/>
-      <c r="L25" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="M25" s="16" t="s">
-        <v>100</v>
-      </c>
-      <c r="N25" s="16"/>
-    </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A26" s="15">
-        <f>IF(B26&lt;&gt;"",COUNTA($B$3:B26),"")</f>
-        <v>24</v>
-      </c>
-      <c r="B26" s="26" t="s">
-        <v>63</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="D26" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="E26" s="15">
-        <v>55.41</v>
-      </c>
       <c r="F26" s="15">
-        <v>0</v>
+        <v>8.4700000000000006</v>
       </c>
       <c r="G26" s="15">
         <v>1</v>
@@ -2239,146 +2323,150 @@
       <c r="H26" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I26" s="3" t="s">
-        <v>98</v>
+      <c r="I26" s="8" t="s">
+        <v>141</v>
       </c>
       <c r="J26" s="15">
         <f t="shared" si="1"/>
-        <v>55.41</v>
+        <v>40.369999999999997</v>
       </c>
       <c r="K26" s="15" t="s">
-        <v>97</v>
-      </c>
-      <c r="L26" s="24" t="s">
-        <v>36</v>
+        <v>140</v>
+      </c>
+      <c r="L26" s="23" t="s">
+        <v>10</v>
       </c>
       <c r="M26" s="16" t="s">
-        <v>99</v>
+        <v>142</v>
       </c>
       <c r="N26" s="16"/>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:14">
       <c r="A27" s="15">
-        <f>IF(B27&lt;&gt;"",COUNTA($B$3:B27),"")</f>
-        <v>25</v>
-      </c>
-      <c r="B27" s="13" t="s">
-        <v>65</v>
+        <f>IF(B28&lt;&gt;"",COUNTA($B$3:B28),"")</f>
+        <v>26</v>
+      </c>
+      <c r="B27" s="25" t="s">
+        <v>63</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="E27" s="15"/>
-      <c r="F27" s="15"/>
+        <v>28</v>
+      </c>
+      <c r="E27" s="15">
+        <v>53.49</v>
+      </c>
+      <c r="F27" s="15">
+        <v>0</v>
+      </c>
       <c r="G27" s="15">
         <v>1</v>
       </c>
       <c r="H27" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I27" s="3"/>
+      <c r="I27" s="8" t="s">
+        <v>143</v>
+      </c>
       <c r="J27" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K27" s="15"/>
-      <c r="L27" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="M27" s="16"/>
+        <v>53.49</v>
+      </c>
+      <c r="K27" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="L27" s="23" t="s">
+        <v>10</v>
+      </c>
+      <c r="M27" s="16" t="s">
+        <v>144</v>
+      </c>
       <c r="N27" s="16"/>
     </row>
-    <row r="28" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14">
       <c r="A28" s="15">
-        <f>IF(B28&lt;&gt;"",COUNTA($B$3:B28),"")</f>
-        <v>26</v>
-      </c>
-      <c r="B28" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="C28" s="21" t="s">
-        <v>108</v>
+        <f>IF(B29&lt;&gt;"",COUNTA($B$3:B29),"")</f>
+        <v>27</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>72</v>
       </c>
       <c r="D28" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E28" s="23">
-        <v>6.99</v>
-      </c>
+      <c r="E28" s="15"/>
       <c r="F28" s="15"/>
       <c r="G28" s="15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H28" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I28" s="22" t="s">
-        <v>111</v>
-      </c>
+      <c r="I28" s="3"/>
       <c r="J28" s="15">
-        <f t="shared" ref="J28" si="2">(G28*E28)+F28</f>
-        <v>27.96</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="K28" s="15"/>
-      <c r="L28" s="24" t="s">
+      <c r="L28" s="23" t="s">
         <v>36</v>
       </c>
       <c r="M28" s="16"/>
       <c r="N28" s="16"/>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14">
       <c r="A29" s="15">
-        <f>IF(B29&lt;&gt;"",COUNTA($B$3:B29),"")</f>
-        <v>27</v>
-      </c>
-      <c r="B29" s="21" t="s">
-        <v>112</v>
-      </c>
-      <c r="C29" s="21" t="s">
-        <v>109</v>
+        <f>IF(B30&lt;&gt;"",COUNTA($B$3:B30),"")</f>
+        <v>28</v>
+      </c>
+      <c r="B29" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="C29" s="20" t="s">
+        <v>100</v>
       </c>
       <c r="D29" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E29" s="15">
-        <v>7.19</v>
+      <c r="E29" s="22">
+        <v>6.99</v>
       </c>
       <c r="F29" s="15"/>
       <c r="G29" s="15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H29" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I29" s="22" t="s">
-        <v>110</v>
+      <c r="I29" s="21" t="s">
+        <v>103</v>
       </c>
       <c r="J29" s="15">
-        <f t="shared" ref="J29" si="3">(G29*E29)+F29</f>
-        <v>14.38</v>
+        <f t="shared" ref="J29" si="2">(G29*E29)+F29</f>
+        <v>27.96</v>
       </c>
       <c r="K29" s="15"/>
-      <c r="L29" s="24" t="s">
-        <v>13</v>
+      <c r="L29" s="23" t="s">
+        <v>36</v>
       </c>
       <c r="M29" s="16"/>
-      <c r="N29" s="16" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N29" s="16"/>
+    </row>
+    <row r="30" spans="1:14">
       <c r="A30" s="15">
-        <f>IF(B30&lt;&gt;"",COUNTA($B$3:B30),"")</f>
-        <v>28</v>
-      </c>
-      <c r="B30" s="21" t="s">
-        <v>114</v>
-      </c>
-      <c r="C30" s="21" t="s">
-        <v>109</v>
+        <f>IF(B31&lt;&gt;"",COUNTA($B$3:B31),"")</f>
+        <v>29</v>
+      </c>
+      <c r="B30" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="C30" s="20" t="s">
+        <v>101</v>
       </c>
       <c r="D30" s="15" t="s">
         <v>25</v>
@@ -2393,109 +2481,148 @@
       <c r="H30" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I30" s="22" t="s">
-        <v>110</v>
+      <c r="I30" s="21" t="s">
+        <v>102</v>
       </c>
       <c r="J30" s="15">
-        <f t="shared" ref="J30" si="4">(G30*E30)+F30</f>
+        <f t="shared" ref="J30" si="3">(G30*E30)+F30</f>
         <v>14.38</v>
       </c>
       <c r="K30" s="15"/>
-      <c r="L30" s="24" t="s">
+      <c r="L30" s="23" t="s">
         <v>13</v>
       </c>
       <c r="M30" s="16"/>
       <c r="N30" s="16" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14">
       <c r="A31" s="15">
-        <f>IF(B31&lt;&gt;"",COUNTA($B$3:B31),"")</f>
-        <v>29</v>
-      </c>
-      <c r="B31" s="21" t="s">
-        <v>116</v>
-      </c>
-      <c r="C31" s="21" t="s">
-        <v>117</v>
+        <f>IF(B32&lt;&gt;"",COUNTA($B$3:B32),"")</f>
+        <v>30</v>
+      </c>
+      <c r="B31" s="20" t="s">
+        <v>106</v>
+      </c>
+      <c r="C31" s="20" t="s">
+        <v>101</v>
       </c>
       <c r="D31" s="15" t="s">
         <v>25</v>
       </c>
       <c r="E31" s="15">
-        <v>4.8899999999999997</v>
+        <v>7.19</v>
       </c>
       <c r="F31" s="15"/>
       <c r="G31" s="15">
+        <v>2</v>
+      </c>
+      <c r="H31" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I31" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="J31" s="15">
+        <f t="shared" ref="J31" si="4">(G31*E31)+F31</f>
+        <v>14.38</v>
+      </c>
+      <c r="K31" s="15"/>
+      <c r="L31" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="M31" s="16"/>
+      <c r="N31" s="16" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14">
+      <c r="A32" s="2">
+        <v>30</v>
+      </c>
+      <c r="B32" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="C32" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="D32" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E32" s="15">
+        <v>4.8899999999999997</v>
+      </c>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15">
         <v>1</v>
       </c>
-      <c r="H31" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="I31" s="22" t="s">
-        <v>115</v>
-      </c>
-      <c r="J31" s="15">
-        <f t="shared" ref="J31" si="5">(G31*E31)+F31</f>
+      <c r="H32" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I32" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="J32" s="15">
+        <f t="shared" ref="J32" si="5">(G32*E32)+F32</f>
         <v>4.8899999999999997</v>
       </c>
-      <c r="K31" s="15"/>
-      <c r="L31" s="24" t="s">
+      <c r="K32" s="15"/>
+      <c r="L32" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="M31" s="16"/>
-      <c r="N31" s="16"/>
-    </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="L32" s="24"/>
-    </row>
-    <row r="33" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L33" s="24"/>
-    </row>
-    <row r="34" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L34" s="24"/>
-    </row>
-    <row r="35" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L35" s="24"/>
-    </row>
-    <row r="36" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L36" s="24"/>
-    </row>
-    <row r="37" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L37" s="24"/>
-    </row>
-    <row r="38" spans="12:12" x14ac:dyDescent="0.3">
-      <c r="L38" s="24"/>
+      <c r="M32" s="16"/>
+      <c r="N32" s="16"/>
+    </row>
+    <row r="33" spans="12:12">
+      <c r="L33" s="23"/>
+    </row>
+    <row r="34" spans="12:12">
+      <c r="L34" s="23"/>
+    </row>
+    <row r="35" spans="12:12">
+      <c r="L35" s="23"/>
+    </row>
+    <row r="36" spans="12:12">
+      <c r="L36" s="23"/>
+    </row>
+    <row r="37" spans="12:12">
+      <c r="L37" s="23"/>
+    </row>
+    <row r="38" spans="12:12">
+      <c r="L38" s="23"/>
+    </row>
+    <row r="39" spans="12:12">
+      <c r="L39" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="F7:F8"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
-  <conditionalFormatting sqref="L3:L6 L10:L38">
-    <cfRule type="containsText" dxfId="5" priority="1" operator="containsText" text="pending">
+  <conditionalFormatting sqref="L3:L6 L10:L12 L14:L39">
+    <cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="pending">
       <formula>NOT(ISERROR(SEARCH("pending",L3)))</formula>
     </cfRule>
     <cfRule type="expression" priority="7">
       <formula>$B2="approved"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L3:L38">
-    <cfRule type="containsText" dxfId="4" priority="3" operator="containsText" text="approved">
+  <conditionalFormatting sqref="L3:L39">
+    <cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="approved">
       <formula>NOT(ISERROR(SEARCH("approved",L3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="ordered">
+    <cfRule type="containsText" dxfId="4" priority="4" operator="containsText" text="ordered">
       <formula>NOT(ISERROR(SEARCH("ordered",L3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="5" operator="containsText" text="rejected">
+    <cfRule type="containsText" dxfId="3" priority="5" operator="containsText" text="rejected">
       <formula>NOT(ISERROR(SEARCH("rejected",L3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="6" operator="containsText" text="received">
+    <cfRule type="containsText" dxfId="2" priority="6" operator="containsText" text="received">
       <formula>NOT(ISERROR(SEARCH("received",L3)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L38">
+  <conditionalFormatting sqref="L4:L39">
     <cfRule type="expression" priority="9">
       <formula>#REF!="approved"</formula>
     </cfRule>
@@ -2506,7 +2633,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L6:L9">
-    <cfRule type="containsText" dxfId="0" priority="12" operator="containsText" text="pending">
+    <cfRule type="containsText" dxfId="1" priority="12" operator="containsText" text="pending">
       <formula>NOT(ISERROR(SEARCH("pending",L6)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2515,15 +2642,28 @@
       <formula>$B5="approved"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="L13">
+    <cfRule type="containsText" dxfId="0" priority="22" operator="containsText" text="pending">
+      <formula>NOT(ISERROR(SEARCH("pending",L13)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="23">
+      <formula>$B11="approved"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <hyperlinks>
     <hyperlink ref="I4" r:id="rId1" display="https://3dprintx.bg/magazin/pa6-cf-with-spool-cherno-bambu-lab/?gad_source=1&amp;gad_campaignid=23369295043&amp;gbraid=0AAAABBeApTZEPbIRHor7bJZ92Gq7vT3lv&amp;gclid=CjwKCAjwxITRBhBYEiwA6mZm7bCe5kvsvoz_znE0dv8i7YoYQrUSTdOaCQ7RKckeGywr-XLrI4hECRoCo7MQAvD_BwE" xr:uid="{45F219EB-CA0E-46B2-B5AC-321500547349}"/>
     <hyperlink ref="I5" r:id="rId2" xr:uid="{29AE6930-3CFD-49FA-8C77-A431B4331D49}"/>
     <hyperlink ref="I6" r:id="rId3" xr:uid="{3002E511-E2F5-4C78-B094-E6DD7CF3B671}"/>
     <hyperlink ref="I7" r:id="rId4" xr:uid="{46C8B073-4590-4C63-B6E5-2A03FB1E94E6}"/>
     <hyperlink ref="I8" r:id="rId5" xr:uid="{7085C41A-4F68-4A70-A26C-EBBC546A59EE}"/>
+    <hyperlink ref="I25" r:id="rId6" xr:uid="{AC3997AD-8B71-448A-BCF4-2A0239242A9A}"/>
+    <hyperlink ref="I19" r:id="rId7" display="https://www.aliexpress.com/item/1005003122596249.html?spm=a2g0o.productlist.main.23.70394477bJf9UQ&amp;algo_pvid=169d2b7f-426b-4582-b7f2-1a69c234abe7&amp;algo_exp_id=169d2b7f-426b-4582-b7f2-1a69c234abe7-20&amp;pdp_ext_f=%7B%22order%22%3A%222145%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%217.69%215.92%21%21%218.62%216.64%21%400b8848e317897611280765333e0f49%2112000024217621966%21sea%21BG%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3Abb4150ed%3Bm03_new_user%3A-29895%3BpisId%3A5000000217831009&amp;curPageLogUid=7PGL6jiPmM9H&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005003122596249%7C_p_origin_prod%3A" xr:uid="{93C2ADC8-BF07-46BD-B25F-9FBD4C8B46B2}"/>
+    <hyperlink ref="I16" r:id="rId8" xr:uid="{1F742A85-6E5F-4512-8BB8-6CC598E9162E}"/>
+    <hyperlink ref="I12" r:id="rId9" xr:uid="{B0912176-1BFC-47C4-867E-D85D256F8603}"/>
+    <hyperlink ref="I27" r:id="rId10" xr:uid="{3AECD8FD-6096-4901-AEEF-DC9E9AE3F865}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId6"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId11"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
@@ -2531,19 +2671,19 @@
           <x14:formula1>
             <xm:f>Background_info!$D$3:$D$30</xm:f>
           </x14:formula1>
-          <xm:sqref>D3:D31</xm:sqref>
+          <xm:sqref>D3:D32</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0CED9412-699B-4C7D-965B-005ACFAE9885}">
           <x14:formula1>
             <xm:f>Background_info!$C$3:$C$15</xm:f>
           </x14:formula1>
-          <xm:sqref>L3:L38</xm:sqref>
+          <xm:sqref>L3:L39</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4580CAC9-FAF7-403B-A1D9-84CB43CB97A9}">
           <x14:formula1>
             <xm:f>Background_info!$B$3:$B$7</xm:f>
           </x14:formula1>
-          <xm:sqref>H3:H31</xm:sqref>
+          <xm:sqref>H3:H32</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2553,18 +2693,359 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F602BA-A80C-4BEA-8ECF-F81C395286C3}">
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:G14"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
-    <col min="2" max="2" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="33" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A1" s="18"/>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="B2" t="s">
-        <v>137</v>
+    <row r="1" spans="1:7">
+      <c r="B1" t="str" cm="1">
+        <f t="array" ref="B1:F1">TRANSPOSE(Background_info!C3:C7)</f>
+        <v>pending</v>
+      </c>
+      <c r="C1" t="str">
+        <v>approved</v>
+      </c>
+      <c r="D1" t="str">
+        <v>ordered</v>
+      </c>
+      <c r="E1" t="str">
+        <v>received</v>
+      </c>
+      <c r="F1" t="str">
+        <v>rejected</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
+        <v>145</v>
+      </c>
+      <c r="B2" s="36">
+        <f>SUM(B3:B14)</f>
+        <v>146.07</v>
+      </c>
+      <c r="C2" s="36">
+        <f t="shared" ref="C2:F2" si="0">SUM(C3:C14)</f>
+        <v>892.29</v>
+      </c>
+      <c r="D2" s="36">
+        <f t="shared" si="0"/>
+        <v>33.32</v>
+      </c>
+      <c r="E2" s="36">
+        <f t="shared" si="0"/>
+        <v>87.460000000000008</v>
+      </c>
+      <c r="F2" s="36">
+        <f t="shared" si="0"/>
+        <v>271.76</v>
+      </c>
+      <c r="G2" s="35">
+        <f>SUM(B2:F2)</f>
+        <v>1430.8999999999999</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
+      <c r="A3" t="str" cm="1">
+        <f t="array" ref="A3:A14">Background_info!D3:D14</f>
+        <v>Airframe and Structures</v>
+      </c>
+      <c r="B3">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A3,Main_Table!$L:$L,B$1)</f>
+        <v>0</v>
+      </c>
+      <c r="C3">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A3,Main_Table!$L:$L,C$1)</f>
+        <v>169.29</v>
+      </c>
+      <c r="D3">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A3,Main_Table!$L:$L,D$1)</f>
+        <v>33.32</v>
+      </c>
+      <c r="E3">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A3,Main_Table!$L:$L,E$1)</f>
+        <v>17.96</v>
+      </c>
+      <c r="F3">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A3,Main_Table!$L:$L,F$1)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4" t="str">
+        <v>Propulsion</v>
+      </c>
+      <c r="B4">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A4,Main_Table!$L:$L,B$1)</f>
+        <v>32.9</v>
+      </c>
+      <c r="C4">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A4,Main_Table!$L:$L,C$1)</f>
+        <v>397.29</v>
+      </c>
+      <c r="D4">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A4,Main_Table!$L:$L,D$1)</f>
+        <v>0</v>
+      </c>
+      <c r="E4">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A4,Main_Table!$L:$L,E$1)</f>
+        <v>0</v>
+      </c>
+      <c r="F4">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A4,Main_Table!$L:$L,F$1)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
+      <c r="A5" t="str">
+        <v>Power</v>
+      </c>
+      <c r="B5">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A5,Main_Table!$L:$L,B$1)</f>
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A5,Main_Table!$L:$L,C$1)</f>
+        <v>190.44</v>
+      </c>
+      <c r="D5">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A5,Main_Table!$L:$L,D$1)</f>
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A5,Main_Table!$L:$L,E$1)</f>
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A5,Main_Table!$L:$L,F$1)</f>
+        <v>243</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
+      <c r="A6" t="str">
+        <v>Flight Control and Avionics</v>
+      </c>
+      <c r="B6">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A6,Main_Table!$L:$L,B$1)</f>
+        <v>32.85</v>
+      </c>
+      <c r="C6">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A6,Main_Table!$L:$L,C$1)</f>
+        <v>63.99</v>
+      </c>
+      <c r="D6">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A6,Main_Table!$L:$L,D$1)</f>
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A6,Main_Table!$L:$L,E$1)</f>
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A6,Main_Table!$L:$L,F$1)</f>
+        <v>28.76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
+      <c r="A7" t="str">
+        <v>Control Surfaces and Mechanisms</v>
+      </c>
+      <c r="B7">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A7,Main_Table!$L:$L,B$1)</f>
+        <v>0</v>
+      </c>
+      <c r="C7">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A7,Main_Table!$L:$L,C$1)</f>
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A7,Main_Table!$L:$L,D$1)</f>
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A7,Main_Table!$L:$L,E$1)</f>
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A7,Main_Table!$L:$L,F$1)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
+      <c r="A8" t="str">
+        <v>Payload and Medical Transport System</v>
+      </c>
+      <c r="B8">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A8,Main_Table!$L:$L,B$1)</f>
+        <v>0</v>
+      </c>
+      <c r="C8">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A8,Main_Table!$L:$L,C$1)</f>
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A8,Main_Table!$L:$L,D$1)</f>
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A8,Main_Table!$L:$L,E$1)</f>
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A8,Main_Table!$L:$L,F$1)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
+      <c r="A9" t="str">
+        <v>Communications and Ground Equipment</v>
+      </c>
+      <c r="B9">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A9,Main_Table!$L:$L,B$1)</f>
+        <v>0</v>
+      </c>
+      <c r="C9">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A9,Main_Table!$L:$L,C$1)</f>
+        <v>53.49</v>
+      </c>
+      <c r="D9">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A9,Main_Table!$L:$L,D$1)</f>
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A9,Main_Table!$L:$L,E$1)</f>
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A9,Main_Table!$L:$L,F$1)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
+      <c r="A10" t="str">
+        <v>Manufacturing and prototyping</v>
+      </c>
+      <c r="B10">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A10,Main_Table!$L:$L,B$1)</f>
+        <v>43.2</v>
+      </c>
+      <c r="C10">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A10,Main_Table!$L:$L,C$1)</f>
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A10,Main_Table!$L:$L,D$1)</f>
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A10,Main_Table!$L:$L,E$1)</f>
+        <v>69.5</v>
+      </c>
+      <c r="F10">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A10,Main_Table!$L:$L,F$1)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
+      <c r="A11" t="str">
+        <v>Fasteners and Consumables</v>
+      </c>
+      <c r="B11">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A11,Main_Table!$L:$L,B$1)</f>
+        <v>37.120000000000005</v>
+      </c>
+      <c r="C11">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A11,Main_Table!$L:$L,C$1)</f>
+        <v>17.79</v>
+      </c>
+      <c r="D11">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A11,Main_Table!$L:$L,D$1)</f>
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A11,Main_Table!$L:$L,E$1)</f>
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A11,Main_Table!$L:$L,F$1)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" t="str">
+        <v>Testing and Safety Equipment</v>
+      </c>
+      <c r="B12">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A12,Main_Table!$L:$L,B$1)</f>
+        <v>0</v>
+      </c>
+      <c r="C12">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A12,Main_Table!$L:$L,C$1)</f>
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A12,Main_Table!$L:$L,D$1)</f>
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A12,Main_Table!$L:$L,E$1)</f>
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A12,Main_Table!$L:$L,F$1)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7">
+      <c r="A13" t="str">
+        <v>Business</v>
+      </c>
+      <c r="B13">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A13,Main_Table!$L:$L,B$1)</f>
+        <v>0</v>
+      </c>
+      <c r="C13">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A13,Main_Table!$L:$L,C$1)</f>
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A13,Main_Table!$L:$L,D$1)</f>
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A13,Main_Table!$L:$L,E$1)</f>
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A13,Main_Table!$L:$L,F$1)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7">
+      <c r="A14" t="str">
+        <v>Other</v>
+      </c>
+      <c r="B14">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A14,Main_Table!$L:$L,B$1)</f>
+        <v>0</v>
+      </c>
+      <c r="C14">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A14,Main_Table!$L:$L,C$1)</f>
+        <v>0</v>
+      </c>
+      <c r="D14">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A14,Main_Table!$L:$L,D$1)</f>
+        <v>0</v>
+      </c>
+      <c r="E14">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A14,Main_Table!$L:$L,E$1)</f>
+        <v>0</v>
+      </c>
+      <c r="F14">
+        <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A14,Main_Table!$L:$L,F$1)</f>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
BOM Update - Adding 8A Ovonic
</commit_message>
<xml_diff>
--- a/P01/P01_06_Procurement/Table_260719_BOM.xlsx
+++ b/P01/P01_06_Procurement/Table_260719_BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10914"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\ORGOfly\ORGOfly-CAD-model\P01\P01_06_Procurement\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martin/Documents/GitHub/ORGOfly-CAD-model/P01/P01_06_Procurement/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DAC9899-B003-4074-BB18-71E93D38844D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A63EB3AE-52E5-A04C-82D7-4F09B24C83FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{EEE73C29-3BDB-49EB-9C57-2FAD514C20AA}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{EEE73C29-3BDB-49EB-9C57-2FAD514C20AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Background_info" sheetId="2" state="hidden" r:id="rId1"/>
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="255" uniqueCount="146">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="148">
   <si>
     <t>#</t>
   </si>
@@ -252,9 +252,6 @@
   </si>
   <si>
     <t>TBS Crossfire Diversity Nano Rx</t>
-  </si>
-  <si>
-    <t>FPV LONG RANGE DRONE RECEIVER</t>
   </si>
   <si>
     <t>ULTRA 25-1600mW 4.9-5.8G 64CH</t>
@@ -503,13 +500,22 @@
   </si>
   <si>
     <t>TOTAL</t>
+  </si>
+  <si>
+    <t>https://www.ampow.com/products/ovonic-roam-series-6s-lipo-battery-8000mah-6s1p-150c-22-2v-lipo-battery-with-xt90-s-anti-spark-plug-for-dji-uav-drone-x-class-6s-hd-cinelifter-long-range</t>
+  </si>
+  <si>
+    <t>Ovonic Roam 6S 8Ah 150C</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -679,7 +685,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -758,23 +764,33 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="7">
+  <dxfs count="8">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -1161,12 +1177,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B02F099F-610B-4C2F-A80F-3888BDD56E8E}">
   <dimension ref="B2:D14"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="4" max="4" width="33.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" ht="15">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
@@ -1177,7 +1193,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="2:4">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>4</v>
       </c>
@@ -1188,7 +1204,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="2:4">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>6</v>
       </c>
@@ -1199,7 +1215,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:4">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>5</v>
       </c>
@@ -1210,7 +1226,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="2:4">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>7</v>
       </c>
@@ -1221,9 +1237,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="2:4">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C7" t="s">
         <v>13</v>
@@ -1232,37 +1248,37 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="2:4">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="2:4">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D9" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="2:4">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="2:4">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D11" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:4">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="2:4">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="2:4">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D14" t="s">
         <v>21</v>
       </c>
@@ -1274,33 +1290,33 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E734346-BCBC-4D9C-B399-F93315446069}">
-  <dimension ref="A1:N39"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
+  <dimension ref="A1:N40"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="30.5" style="7" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="50" style="2" customWidth="1"/>
-    <col min="4" max="4" width="37.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="8.875" style="1"/>
-    <col min="7" max="7" width="8.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.375" style="1" customWidth="1"/>
+    <col min="4" max="4" width="37.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="8.83203125" style="1"/>
+    <col min="7" max="7" width="8.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.33203125" style="1" customWidth="1"/>
     <col min="11" max="11" width="9.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.875" style="1"/>
+    <col min="12" max="12" width="8.83203125" style="1"/>
     <col min="13" max="13" width="55" style="17" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="60.75" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.875" style="2"/>
+    <col min="14" max="14" width="60.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C1" s="6"/>
       <c r="M1" s="2"/>
     </row>
-    <row r="2" spans="1:14" ht="27" customHeight="1">
+    <row r="2" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
@@ -1341,10 +1357,10 @@
         <v>14</v>
       </c>
       <c r="N2" s="11" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="15">
         <f>IF(B3&lt;&gt;"",COUNTA($B$3:B3),"")</f>
         <v>1</v>
@@ -1382,7 +1398,7 @@
       <c r="M3" s="16"/>
       <c r="N3" s="16"/>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="15">
         <f>IF(B4&lt;&gt;"",COUNTA($B$3:B4),"")</f>
         <v>2</v>
@@ -1426,16 +1442,16 @@
       </c>
       <c r="N4" s="16"/>
     </row>
-    <row r="5" spans="1:14" ht="28.5">
+    <row r="5" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="15">
         <f>IF(B5&lt;&gt;"",COUNTA($B$3:B5),"")</f>
         <v>3</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>24</v>
@@ -1450,27 +1466,27 @@
         <v>1</v>
       </c>
       <c r="H5" s="15" t="s">
+        <v>115</v>
+      </c>
+      <c r="I5" s="8" t="s">
         <v>116</v>
-      </c>
-      <c r="I5" s="8" t="s">
-        <v>117</v>
       </c>
       <c r="J5" s="15">
         <f>(G5*E5)+F5</f>
         <v>17.96</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L5" s="23" t="s">
         <v>12</v>
       </c>
       <c r="M5" s="18" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="N5" s="16"/>
     </row>
-    <row r="6" spans="1:14" ht="42.75">
+    <row r="6" spans="1:14" ht="48" x14ac:dyDescent="0.2">
       <c r="A6" s="15">
         <f>IF(B6&lt;&gt;"",COUNTA($B$3:B6),"")</f>
         <v>4</v>
@@ -1479,7 +1495,7 @@
         <v>40</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>24</v>
@@ -1494,27 +1510,27 @@
         <v>1</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J6" s="15">
         <f>(G6*E6)+F6</f>
         <v>33.32</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="L6" s="23" t="s">
         <v>11</v>
       </c>
       <c r="M6" s="18" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="N6" s="16"/>
     </row>
-    <row r="7" spans="1:14" ht="28.5">
+    <row r="7" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="15">
         <f>IF(B7&lt;&gt;"",COUNTA($B$3:B7),"")</f>
         <v>5</v>
@@ -1531,7 +1547,7 @@
       <c r="E7" s="15">
         <v>31.22</v>
       </c>
-      <c r="F7" s="32">
+      <c r="F7" s="35">
         <v>18.75</v>
       </c>
       <c r="G7" s="15">
@@ -1541,24 +1557,24 @@
         <v>4</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="J7" s="15">
-        <f t="shared" ref="J7:J22" si="0">(G7*E7)+F7</f>
+        <f t="shared" ref="J7:J23" si="0">(G7*E7)+F7</f>
         <v>143.63</v>
       </c>
       <c r="K7" s="24" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="L7" s="23" t="s">
         <v>10</v>
       </c>
       <c r="M7" s="18" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N7" s="16"/>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="15">
         <f>IF(B8&lt;&gt;"",COUNTA($B$3:B8),"")</f>
         <v>6</v>
@@ -1575,7 +1591,7 @@
       <c r="E8" s="15">
         <v>12.83</v>
       </c>
-      <c r="F8" s="33"/>
+      <c r="F8" s="36"/>
       <c r="G8" s="15">
         <v>2</v>
       </c>
@@ -1583,24 +1599,24 @@
         <v>4</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="J8" s="15">
         <f t="shared" si="0"/>
         <v>25.66</v>
       </c>
       <c r="K8" s="24" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="L8" s="23" t="s">
         <v>10</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="N8" s="16"/>
     </row>
-    <row r="9" spans="1:14" ht="28.5">
+    <row r="9" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="15">
         <f>IF(B9&lt;&gt;"",COUNTA($B$3:B9),"")</f>
         <v>7</v>
@@ -1627,7 +1643,7 @@
         <v>4</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J9" s="15">
         <f t="shared" si="0"/>
@@ -1640,11 +1656,11 @@
         <v>12</v>
       </c>
       <c r="M9" s="18" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N9" s="31"/>
     </row>
-    <row r="10" spans="1:14" ht="15">
+    <row r="10" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="15">
         <f>IF(B10&lt;&gt;"",COUNTA($B$3:B10),"")</f>
         <v>8</v>
@@ -1677,12 +1693,12 @@
       <c r="M10" s="16"/>
       <c r="N10" s="16"/>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="15">
         <f>IF(B11&lt;&gt;"",COUNTA($B$3:B11),"")</f>
         <v>9</v>
       </c>
-      <c r="B11" s="34" t="s">
+      <c r="B11" s="32" t="s">
         <v>57</v>
       </c>
       <c r="C11" s="13" t="s">
@@ -1704,32 +1720,29 @@
         <v>4</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="J11" s="15">
         <f t="shared" si="0"/>
         <v>243</v>
       </c>
       <c r="K11" s="15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="L11" s="23" t="s">
         <v>13</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="N11" s="16" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
-      <c r="A12" s="15">
-        <f>IF(B13&lt;&gt;"",COUNTA($B$3:B13),"")</f>
-        <v>11</v>
-      </c>
+        <v>128</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="15"/>
       <c r="B12" s="28" t="s">
-        <v>131</v>
+        <v>146</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>51</v>
@@ -1738,54 +1751,39 @@
         <v>19</v>
       </c>
       <c r="E12" s="15">
-        <v>62.75</v>
-      </c>
-      <c r="F12" s="15">
-        <v>24.57</v>
-      </c>
-      <c r="G12" s="15">
-        <v>2</v>
-      </c>
-      <c r="H12" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="I12" s="8" t="s">
-        <v>133</v>
-      </c>
-      <c r="J12" s="15">
-        <f t="shared" si="0"/>
-        <v>150.07</v>
-      </c>
-      <c r="K12" s="24" t="s">
-        <v>132</v>
-      </c>
-      <c r="L12" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="M12" s="16" t="s">
-        <v>130</v>
-      </c>
+        <v>92</v>
+      </c>
+      <c r="F12" s="15"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="37" t="s">
+        <v>145</v>
+      </c>
+      <c r="J12" s="15"/>
+      <c r="K12" s="15"/>
+      <c r="L12" s="23"/>
+      <c r="M12" s="16"/>
       <c r="N12" s="16"/>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="15">
         <f>IF(B14&lt;&gt;"",COUNTA($B$3:B14),"")</f>
         <v>12</v>
       </c>
-      <c r="B13" s="26" t="s">
-        <v>97</v>
+      <c r="B13" s="28" t="s">
+        <v>130</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="E13" s="15">
-        <v>16.45</v>
+        <v>62.75</v>
       </c>
       <c r="F13" s="15">
-        <v>0</v>
+        <v>24.57</v>
       </c>
       <c r="G13" s="15">
         <v>2</v>
@@ -1793,71 +1791,81 @@
       <c r="H13" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I13" s="3" t="s">
-        <v>96</v>
+      <c r="I13" s="8" t="s">
+        <v>132</v>
       </c>
       <c r="J13" s="15">
         <f t="shared" si="0"/>
-        <v>32.9</v>
-      </c>
-      <c r="K13" s="15" t="s">
-        <v>48</v>
+        <v>150.07</v>
+      </c>
+      <c r="K13" s="24" t="s">
+        <v>131</v>
       </c>
       <c r="L13" s="23" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="M13" s="16" t="s">
-        <v>98</v>
+        <v>129</v>
       </c>
       <c r="N13" s="16"/>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="15">
         <f>IF(B15&lt;&gt;"",COUNTA($B$3:B15),"")</f>
         <v>13</v>
       </c>
-      <c r="B14" s="34" t="s">
-        <v>56</v>
+      <c r="B14" s="26" t="s">
+        <v>96</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>52</v>
+        <v>94</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>19</v>
-      </c>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
+        <v>18</v>
+      </c>
+      <c r="E14" s="15">
+        <v>16.45</v>
+      </c>
+      <c r="F14" s="15">
+        <v>0</v>
+      </c>
       <c r="G14" s="15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H14" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I14" s="3"/>
+      <c r="I14" s="8" t="s">
+        <v>95</v>
+      </c>
       <c r="J14" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K14" s="15"/>
+        <v>32.9</v>
+      </c>
+      <c r="K14" s="15" t="s">
+        <v>48</v>
+      </c>
       <c r="L14" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="M14" s="16"/>
+      <c r="M14" s="16" t="s">
+        <v>97</v>
+      </c>
       <c r="N14" s="16"/>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="15">
         <f>IF(B16&lt;&gt;"",COUNTA($B$3:B16),"")</f>
         <v>14</v>
       </c>
-      <c r="B15" s="13" t="s">
-        <v>58</v>
+      <c r="B15" s="32" t="s">
+        <v>56</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="E15" s="15"/>
       <c r="F15" s="15"/>
@@ -1879,179 +1887,169 @@
       <c r="M15" s="16"/>
       <c r="N15" s="16"/>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="15">
         <f>IF(B17&lt;&gt;"",COUNTA($B$3:B17),"")</f>
         <v>15</v>
       </c>
-      <c r="B16" s="28" t="s">
-        <v>53</v>
+      <c r="B16" s="13" t="s">
+        <v>58</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>71</v>
+        <v>59</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E16" s="15">
-        <v>51.39</v>
-      </c>
-      <c r="F16" s="15">
-        <v>16.739999999999998</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
       <c r="G16" s="15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H16" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I16" s="8" t="s">
-        <v>134</v>
-      </c>
+      <c r="I16" s="3"/>
       <c r="J16" s="15">
         <f t="shared" si="0"/>
-        <v>222.3</v>
-      </c>
-      <c r="K16" s="15" t="s">
-        <v>94</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K16" s="15"/>
       <c r="L16" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="M16" s="16" t="s">
-        <v>135</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="M16" s="16"/>
       <c r="N16" s="16"/>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="15">
         <f>IF(B18&lt;&gt;"",COUNTA($B$3:B18),"")</f>
         <v>16</v>
       </c>
       <c r="B17" s="28" t="s">
-        <v>69</v>
+        <v>53</v>
       </c>
       <c r="C17" s="13" t="s">
         <v>70</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="E17" s="15">
-        <v>63.99</v>
+        <v>51.39</v>
       </c>
       <c r="F17" s="15">
-        <v>0</v>
+        <v>16.739999999999998</v>
       </c>
       <c r="G17" s="15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H17" s="15" t="s">
         <v>4</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="J17" s="15">
         <f t="shared" si="0"/>
-        <v>63.99</v>
+        <v>222.3</v>
       </c>
       <c r="K17" s="15" t="s">
-        <v>137</v>
+        <v>93</v>
       </c>
       <c r="L17" s="23" t="s">
         <v>10</v>
       </c>
       <c r="M17" s="16" t="s">
-        <v>93</v>
+        <v>134</v>
       </c>
       <c r="N17" s="16"/>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="15">
         <f>IF(B19&lt;&gt;"",COUNTA($B$3:B19),"")</f>
         <v>17</v>
       </c>
-      <c r="B18" s="26" t="s">
-        <v>54</v>
+      <c r="B18" s="28" t="s">
+        <v>68</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15"/>
+      <c r="E18" s="15">
+        <v>63.99</v>
+      </c>
+      <c r="F18" s="15">
+        <v>0</v>
+      </c>
       <c r="G18" s="15">
         <v>1</v>
       </c>
       <c r="H18" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I18" s="3"/>
+      <c r="I18" s="8" t="s">
+        <v>135</v>
+      </c>
       <c r="J18" s="15">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K18" s="15"/>
+        <v>63.99</v>
+      </c>
+      <c r="K18" s="15" t="s">
+        <v>136</v>
+      </c>
       <c r="L18" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="M18" s="16"/>
+        <v>10</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>92</v>
+      </c>
       <c r="N18" s="16"/>
     </row>
-    <row r="19" spans="1:14" ht="28.5">
+    <row r="19" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="15">
         <f>IF(B20&lt;&gt;"",COUNTA($B$3:B20),"")</f>
         <v>18</v>
       </c>
-      <c r="B19" s="28" t="s">
-        <v>75</v>
+      <c r="B19" s="26" t="s">
+        <v>54</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="D19" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="E19" s="15">
-        <v>5.92</v>
-      </c>
-      <c r="F19" s="15">
-        <v>5.95</v>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="E19" s="15"/>
+      <c r="F19" s="15"/>
       <c r="G19" s="15">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H19" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I19" s="8" t="s">
-        <v>139</v>
-      </c>
+      <c r="I19" s="3"/>
       <c r="J19" s="15">
         <f t="shared" si="0"/>
-        <v>17.79</v>
-      </c>
-      <c r="K19" s="15" t="s">
-        <v>137</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K19" s="15"/>
       <c r="L19" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="M19" s="16" t="s">
-        <v>138</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="M19" s="16"/>
       <c r="N19" s="16"/>
     </row>
-    <row r="20" spans="1:14" ht="28.5">
+    <row r="20" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" s="15">
         <f>IF(B21&lt;&gt;"",COUNTA($B$3:B21),"")</f>
         <v>19</v>
       </c>
-      <c r="B20" s="26" t="s">
-        <v>77</v>
+      <c r="B20" s="28" t="s">
+        <v>74</v>
       </c>
       <c r="C20" s="13" t="s">
         <v>60</v>
@@ -2060,51 +2058,51 @@
         <v>30</v>
       </c>
       <c r="E20" s="15">
-        <v>7.04</v>
+        <v>5.92</v>
       </c>
       <c r="F20" s="15">
-        <v>0</v>
+        <v>5.95</v>
       </c>
       <c r="G20" s="15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H20" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I20" s="3" t="s">
-        <v>78</v>
+      <c r="I20" s="8" t="s">
+        <v>138</v>
       </c>
       <c r="J20" s="15">
         <f t="shared" si="0"/>
-        <v>7.04</v>
+        <v>17.79</v>
       </c>
       <c r="K20" s="15" t="s">
-        <v>48</v>
+        <v>136</v>
       </c>
       <c r="L20" s="23" t="s">
-        <v>36</v>
+        <v>10</v>
       </c>
       <c r="M20" s="16" t="s">
-        <v>76</v>
+        <v>137</v>
       </c>
       <c r="N20" s="16"/>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A21" s="15">
         <f>IF(B22&lt;&gt;"",COUNTA($B$3:B22),"")</f>
         <v>20</v>
       </c>
       <c r="B21" s="26" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>86</v>
+        <v>60</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>30</v>
       </c>
       <c r="E21" s="15">
-        <v>14.81</v>
+        <v>7.04</v>
       </c>
       <c r="F21" s="15">
         <v>0</v>
@@ -2116,11 +2114,11 @@
         <v>4</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="J21" s="15">
         <f t="shared" si="0"/>
-        <v>14.81</v>
+        <v>7.04</v>
       </c>
       <c r="K21" s="15" t="s">
         <v>48</v>
@@ -2129,17 +2127,17 @@
         <v>36</v>
       </c>
       <c r="M21" s="16" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="N21" s="16"/>
     </row>
-    <row r="22" spans="1:14">
+    <row r="22" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="15">
         <f>IF(B23&lt;&gt;"",COUNTA($B$3:B23),"")</f>
         <v>21</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>87</v>
+        <v>78</v>
       </c>
       <c r="C22" s="13" t="s">
         <v>85</v>
@@ -2148,7 +2146,7 @@
         <v>30</v>
       </c>
       <c r="E22" s="15">
-        <v>6.61</v>
+        <v>14.81</v>
       </c>
       <c r="F22" s="15">
         <v>0</v>
@@ -2160,11 +2158,11 @@
         <v>4</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="J22" s="15">
         <f t="shared" si="0"/>
-        <v>6.61</v>
+        <v>14.81</v>
       </c>
       <c r="K22" s="15" t="s">
         <v>48</v>
@@ -2173,26 +2171,26 @@
         <v>36</v>
       </c>
       <c r="M22" s="16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="N22" s="16"/>
     </row>
-    <row r="23" spans="1:14" ht="12.75" customHeight="1">
+    <row r="23" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="15">
         <f>IF(B24&lt;&gt;"",COUNTA($B$3:B24),"")</f>
         <v>22</v>
       </c>
-      <c r="B23" s="29" t="s">
-        <v>81</v>
+      <c r="B23" s="26" t="s">
+        <v>86</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D23" s="15" t="s">
         <v>30</v>
       </c>
       <c r="E23" s="15">
-        <v>8.66</v>
+        <v>6.61</v>
       </c>
       <c r="F23" s="15">
         <v>0</v>
@@ -2203,12 +2201,12 @@
       <c r="H23" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I23" s="13" t="s">
-        <v>80</v>
+      <c r="I23" s="3" t="s">
+        <v>83</v>
       </c>
       <c r="J23" s="15">
-        <f t="shared" ref="J23:J28" si="1">(G23*E23)+F23</f>
-        <v>8.66</v>
+        <f t="shared" si="0"/>
+        <v>6.61</v>
       </c>
       <c r="K23" s="15" t="s">
         <v>48</v>
@@ -2216,106 +2214,106 @@
       <c r="L23" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="M23" s="16"/>
+      <c r="M23" s="16" t="s">
+        <v>73</v>
+      </c>
       <c r="N23" s="16"/>
     </row>
-    <row r="24" spans="1:14" ht="15">
+    <row r="24" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="15">
         <f>IF(B25&lt;&gt;"",COUNTA($B$3:B25),"")</f>
         <v>23</v>
       </c>
-      <c r="B24" s="19" t="s">
-        <v>61</v>
+      <c r="B24" s="29" t="s">
+        <v>80</v>
       </c>
       <c r="C24" s="13" t="s">
-        <v>55</v>
+        <v>81</v>
       </c>
       <c r="D24" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="E24" s="15"/>
-      <c r="F24" s="15"/>
+      <c r="E24" s="15">
+        <v>8.66</v>
+      </c>
+      <c r="F24" s="15">
+        <v>0</v>
+      </c>
       <c r="G24" s="15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H24" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I24" s="3"/>
+      <c r="I24" s="13" t="s">
+        <v>79</v>
+      </c>
       <c r="J24" s="15">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K24" s="15"/>
+        <f t="shared" ref="J24:J29" si="1">(G24*E24)+F24</f>
+        <v>8.66</v>
+      </c>
+      <c r="K24" s="15" t="s">
+        <v>48</v>
+      </c>
       <c r="L24" s="23" t="s">
         <v>36</v>
       </c>
       <c r="M24" s="16"/>
       <c r="N24" s="16"/>
     </row>
-    <row r="25" spans="1:14" ht="28.5">
+    <row r="25" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="15">
         <f>IF(B26&lt;&gt;"",COUNTA($B$3:B26),"")</f>
         <v>24</v>
       </c>
-      <c r="B25" s="25" t="s">
-        <v>89</v>
+      <c r="B25" s="19" t="s">
+        <v>61</v>
       </c>
       <c r="C25" s="13" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>18</v>
-      </c>
-      <c r="E25" s="15">
-        <v>174.99</v>
-      </c>
-      <c r="F25" s="15">
-        <v>0</v>
-      </c>
+        <v>30</v>
+      </c>
+      <c r="E25" s="15"/>
+      <c r="F25" s="15"/>
       <c r="G25" s="15">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H25" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I25" s="8" t="s">
-        <v>88</v>
-      </c>
+      <c r="I25" s="3"/>
       <c r="J25" s="15">
         <f t="shared" si="1"/>
-        <v>174.99</v>
-      </c>
-      <c r="K25" s="15" t="s">
-        <v>90</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="K25" s="15"/>
       <c r="L25" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="M25" s="16" t="s">
-        <v>91</v>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="M25" s="16"/>
       <c r="N25" s="16"/>
     </row>
-    <row r="26" spans="1:14">
+    <row r="26" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="15">
         <f>IF(B27&lt;&gt;"",COUNTA($B$3:B27),"")</f>
         <v>25</v>
       </c>
-      <c r="B26" s="30" t="s">
-        <v>66</v>
+      <c r="B26" s="25" t="s">
+        <v>88</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="D26" s="15" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E26" s="15">
-        <v>31.9</v>
+        <v>174.99</v>
       </c>
       <c r="F26" s="15">
-        <v>8.4700000000000006</v>
+        <v>0</v>
       </c>
       <c r="G26" s="15">
         <v>1</v>
@@ -2324,42 +2322,42 @@
         <v>4</v>
       </c>
       <c r="I26" s="8" t="s">
-        <v>141</v>
+        <v>87</v>
       </c>
       <c r="J26" s="15">
         <f t="shared" si="1"/>
-        <v>40.369999999999997</v>
+        <v>174.99</v>
       </c>
       <c r="K26" s="15" t="s">
-        <v>140</v>
+        <v>89</v>
       </c>
       <c r="L26" s="23" t="s">
         <v>10</v>
       </c>
       <c r="M26" s="16" t="s">
-        <v>142</v>
+        <v>90</v>
       </c>
       <c r="N26" s="16"/>
     </row>
-    <row r="27" spans="1:14">
+    <row r="27" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="15">
         <f>IF(B28&lt;&gt;"",COUNTA($B$3:B28),"")</f>
         <v>26</v>
       </c>
-      <c r="B27" s="25" t="s">
-        <v>63</v>
+      <c r="B27" s="30" t="s">
+        <v>65</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D27" s="15" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="E27" s="15">
-        <v>53.49</v>
+        <v>31.9</v>
       </c>
       <c r="F27" s="15">
-        <v>0</v>
+        <v>8.4700000000000006</v>
       </c>
       <c r="G27" s="15">
         <v>1</v>
@@ -2368,87 +2366,93 @@
         <v>4</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="J27" s="15">
         <f t="shared" si="1"/>
-        <v>53.49</v>
+        <v>40.369999999999997</v>
       </c>
       <c r="K27" s="15" t="s">
-        <v>92</v>
+        <v>139</v>
       </c>
       <c r="L27" s="23" t="s">
         <v>10</v>
       </c>
       <c r="M27" s="16" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="N27" s="16"/>
     </row>
-    <row r="28" spans="1:14">
+    <row r="28" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="15">
         <f>IF(B29&lt;&gt;"",COUNTA($B$3:B29),"")</f>
         <v>27</v>
       </c>
-      <c r="B28" s="13" t="s">
-        <v>65</v>
+      <c r="B28" s="25" t="s">
+        <v>63</v>
       </c>
       <c r="C28" s="13" t="s">
-        <v>72</v>
+        <v>147</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="E28" s="15"/>
-      <c r="F28" s="15"/>
+        <v>28</v>
+      </c>
+      <c r="E28" s="15">
+        <v>53.49</v>
+      </c>
+      <c r="F28" s="15">
+        <v>0</v>
+      </c>
       <c r="G28" s="15">
         <v>1</v>
       </c>
       <c r="H28" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I28" s="3"/>
+      <c r="I28" s="8" t="s">
+        <v>142</v>
+      </c>
       <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K28" s="15"/>
+        <v>53.49</v>
+      </c>
+      <c r="K28" s="15" t="s">
+        <v>91</v>
+      </c>
       <c r="L28" s="23" t="s">
-        <v>36</v>
-      </c>
-      <c r="M28" s="16"/>
+        <v>10</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>143</v>
+      </c>
       <c r="N28" s="16"/>
     </row>
-    <row r="29" spans="1:14">
+    <row r="29" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="15">
         <f>IF(B30&lt;&gt;"",COUNTA($B$3:B30),"")</f>
         <v>28</v>
       </c>
-      <c r="B29" s="20" t="s">
-        <v>105</v>
-      </c>
-      <c r="C29" s="20" t="s">
-        <v>100</v>
+      <c r="B29" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>71</v>
       </c>
       <c r="D29" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E29" s="22">
-        <v>6.99</v>
-      </c>
+      <c r="E29" s="15"/>
       <c r="F29" s="15"/>
       <c r="G29" s="15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H29" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I29" s="21" t="s">
-        <v>103</v>
-      </c>
+      <c r="I29" s="3"/>
       <c r="J29" s="15">
-        <f t="shared" ref="J29" si="2">(G29*E29)+F29</f>
-        <v>27.96</v>
+        <f t="shared" si="1"/>
+        <v>0</v>
       </c>
       <c r="K29" s="15"/>
       <c r="L29" s="23" t="s">
@@ -2457,7 +2461,7 @@
       <c r="M29" s="16"/>
       <c r="N29" s="16"/>
     </row>
-    <row r="30" spans="1:14">
+    <row r="30" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="15">
         <f>IF(B31&lt;&gt;"",COUNTA($B$3:B31),"")</f>
         <v>29</v>
@@ -2466,17 +2470,17 @@
         <v>104</v>
       </c>
       <c r="C30" s="20" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D30" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E30" s="15">
-        <v>7.19</v>
+      <c r="E30" s="22">
+        <v>6.99</v>
       </c>
       <c r="F30" s="15"/>
       <c r="G30" s="15">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H30" s="15" t="s">
         <v>4</v>
@@ -2485,28 +2489,26 @@
         <v>102</v>
       </c>
       <c r="J30" s="15">
-        <f t="shared" ref="J30" si="3">(G30*E30)+F30</f>
-        <v>14.38</v>
+        <f t="shared" ref="J30" si="2">(G30*E30)+F30</f>
+        <v>27.96</v>
       </c>
       <c r="K30" s="15"/>
       <c r="L30" s="23" t="s">
-        <v>13</v>
+        <v>36</v>
       </c>
       <c r="M30" s="16"/>
-      <c r="N30" s="16" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="31" spans="1:14">
+      <c r="N30" s="16"/>
+    </row>
+    <row r="31" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="15">
         <f>IF(B32&lt;&gt;"",COUNTA($B$3:B32),"")</f>
         <v>30</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C31" s="20" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D31" s="15" t="s">
         <v>25</v>
@@ -2522,10 +2524,10 @@
         <v>4</v>
       </c>
       <c r="I31" s="21" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J31" s="15">
-        <f t="shared" ref="J31" si="4">(G31*E31)+F31</f>
+        <f t="shared" ref="J31" si="3">(G31*E31)+F31</f>
         <v>14.38</v>
       </c>
       <c r="K31" s="15"/>
@@ -2534,95 +2536,135 @@
       </c>
       <c r="M31" s="16"/>
       <c r="N31" s="16" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="32" spans="1:14">
-      <c r="A32" s="2">
-        <v>30</v>
+        <v>127</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+      <c r="A32" s="15">
+        <f>IF(B33&lt;&gt;"",COUNTA($B$3:B33),"")</f>
+        <v>31</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C32" s="20" t="s">
-        <v>109</v>
+        <v>100</v>
       </c>
       <c r="D32" s="15" t="s">
         <v>25</v>
       </c>
       <c r="E32" s="15">
-        <v>4.8899999999999997</v>
+        <v>7.19</v>
       </c>
       <c r="F32" s="15"/>
       <c r="G32" s="15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H32" s="15" t="s">
         <v>4</v>
       </c>
       <c r="I32" s="21" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="J32" s="15">
-        <f t="shared" ref="J32" si="5">(G32*E32)+F32</f>
-        <v>4.8899999999999997</v>
+        <f t="shared" ref="J32" si="4">(G32*E32)+F32</f>
+        <v>14.38</v>
       </c>
       <c r="K32" s="15"/>
       <c r="L32" s="23" t="s">
+        <v>13</v>
+      </c>
+      <c r="M32" s="16"/>
+      <c r="N32" s="16" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+      <c r="A33" s="2">
+        <v>30</v>
+      </c>
+      <c r="B33" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="C33" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E33" s="15">
+        <v>4.8899999999999997</v>
+      </c>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15">
+        <v>1</v>
+      </c>
+      <c r="H33" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I33" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="J33" s="15">
+        <f t="shared" ref="J33" si="5">(G33*E33)+F33</f>
+        <v>4.8899999999999997</v>
+      </c>
+      <c r="K33" s="15"/>
+      <c r="L33" s="23" t="s">
         <v>36</v>
       </c>
-      <c r="M32" s="16"/>
-      <c r="N32" s="16"/>
-    </row>
-    <row r="33" spans="12:12">
-      <c r="L33" s="23"/>
-    </row>
-    <row r="34" spans="12:12">
+      <c r="M33" s="16"/>
+      <c r="N33" s="16"/>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.2">
       <c r="L34" s="23"/>
     </row>
-    <row r="35" spans="12:12">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.2">
       <c r="L35" s="23"/>
     </row>
-    <row r="36" spans="12:12">
+    <row r="36" spans="1:14" x14ac:dyDescent="0.2">
       <c r="L36" s="23"/>
     </row>
-    <row r="37" spans="12:12">
+    <row r="37" spans="1:14" x14ac:dyDescent="0.2">
       <c r="L37" s="23"/>
     </row>
-    <row r="38" spans="12:12">
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
       <c r="L38" s="23"/>
     </row>
-    <row r="39" spans="12:12">
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
       <c r="L39" s="23"/>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="L40" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="F7:F8"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
-  <conditionalFormatting sqref="L3:L6 L10:L12 L14:L39">
-    <cfRule type="containsText" dxfId="6" priority="1" operator="containsText" text="pending">
+  <conditionalFormatting sqref="L3:L6 L15:L40 L10:L12">
+    <cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="pending">
       <formula>NOT(ISERROR(SEARCH("pending",L3)))</formula>
     </cfRule>
     <cfRule type="expression" priority="7">
       <formula>$B2="approved"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L3:L39">
-    <cfRule type="containsText" dxfId="5" priority="3" operator="containsText" text="approved">
+  <conditionalFormatting sqref="L3:L40">
+    <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="approved">
       <formula>NOT(ISERROR(SEARCH("approved",L3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="4" priority="4" operator="containsText" text="ordered">
+    <cfRule type="containsText" dxfId="5" priority="4" operator="containsText" text="ordered">
       <formula>NOT(ISERROR(SEARCH("ordered",L3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="5" operator="containsText" text="rejected">
+    <cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="rejected">
       <formula>NOT(ISERROR(SEARCH("rejected",L3)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="6" operator="containsText" text="received">
+    <cfRule type="containsText" dxfId="3" priority="6" operator="containsText" text="received">
       <formula>NOT(ISERROR(SEARCH("received",L3)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L39">
+  <conditionalFormatting sqref="L4:L40">
     <cfRule type="expression" priority="9">
       <formula>#REF!="approved"</formula>
     </cfRule>
@@ -2633,7 +2675,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L6:L9">
-    <cfRule type="containsText" dxfId="1" priority="12" operator="containsText" text="pending">
+    <cfRule type="containsText" dxfId="2" priority="12" operator="containsText" text="pending">
       <formula>NOT(ISERROR(SEARCH("pending",L6)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2642,11 +2684,19 @@
       <formula>$B5="approved"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="L14">
+    <cfRule type="containsText" dxfId="1" priority="22" operator="containsText" text="pending">
+      <formula>NOT(ISERROR(SEARCH("pending",L14)))</formula>
+    </cfRule>
+    <cfRule type="expression" priority="23">
+      <formula>$B11="approved"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L13">
-    <cfRule type="containsText" dxfId="0" priority="22" operator="containsText" text="pending">
+    <cfRule type="containsText" dxfId="0" priority="26" operator="containsText" text="pending">
       <formula>NOT(ISERROR(SEARCH("pending",L13)))</formula>
     </cfRule>
-    <cfRule type="expression" priority="23">
+    <cfRule type="expression" priority="27">
       <formula>$B11="approved"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -2656,14 +2706,17 @@
     <hyperlink ref="I6" r:id="rId3" xr:uid="{3002E511-E2F5-4C78-B094-E6DD7CF3B671}"/>
     <hyperlink ref="I7" r:id="rId4" xr:uid="{46C8B073-4590-4C63-B6E5-2A03FB1E94E6}"/>
     <hyperlink ref="I8" r:id="rId5" xr:uid="{7085C41A-4F68-4A70-A26C-EBBC546A59EE}"/>
-    <hyperlink ref="I25" r:id="rId6" xr:uid="{AC3997AD-8B71-448A-BCF4-2A0239242A9A}"/>
-    <hyperlink ref="I19" r:id="rId7" display="https://www.aliexpress.com/item/1005003122596249.html?spm=a2g0o.productlist.main.23.70394477bJf9UQ&amp;algo_pvid=169d2b7f-426b-4582-b7f2-1a69c234abe7&amp;algo_exp_id=169d2b7f-426b-4582-b7f2-1a69c234abe7-20&amp;pdp_ext_f=%7B%22order%22%3A%222145%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%217.69%215.92%21%21%218.62%216.64%21%400b8848e317897611280765333e0f49%2112000024217621966%21sea%21BG%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3Abb4150ed%3Bm03_new_user%3A-29895%3BpisId%3A5000000217831009&amp;curPageLogUid=7PGL6jiPmM9H&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005003122596249%7C_p_origin_prod%3A" xr:uid="{93C2ADC8-BF07-46BD-B25F-9FBD4C8B46B2}"/>
-    <hyperlink ref="I16" r:id="rId8" xr:uid="{1F742A85-6E5F-4512-8BB8-6CC598E9162E}"/>
-    <hyperlink ref="I12" r:id="rId9" xr:uid="{B0912176-1BFC-47C4-867E-D85D256F8603}"/>
-    <hyperlink ref="I27" r:id="rId10" xr:uid="{3AECD8FD-6096-4901-AEEF-DC9E9AE3F865}"/>
+    <hyperlink ref="I26" r:id="rId6" xr:uid="{AC3997AD-8B71-448A-BCF4-2A0239242A9A}"/>
+    <hyperlink ref="I20" r:id="rId7" display="https://www.aliexpress.com/item/1005003122596249.html?spm=a2g0o.productlist.main.23.70394477bJf9UQ&amp;algo_pvid=169d2b7f-426b-4582-b7f2-1a69c234abe7&amp;algo_exp_id=169d2b7f-426b-4582-b7f2-1a69c234abe7-20&amp;pdp_ext_f=%7B%22order%22%3A%222145%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%217.69%215.92%21%21%218.62%216.64%21%400b8848e317897611280765333e0f49%2112000024217621966%21sea%21BG%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3Abb4150ed%3Bm03_new_user%3A-29895%3BpisId%3A5000000217831009&amp;curPageLogUid=7PGL6jiPmM9H&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005003122596249%7C_p_origin_prod%3A" xr:uid="{93C2ADC8-BF07-46BD-B25F-9FBD4C8B46B2}"/>
+    <hyperlink ref="I17" r:id="rId8" xr:uid="{1F742A85-6E5F-4512-8BB8-6CC598E9162E}"/>
+    <hyperlink ref="I13" r:id="rId9" xr:uid="{B0912176-1BFC-47C4-867E-D85D256F8603}"/>
+    <hyperlink ref="I28" r:id="rId10" xr:uid="{3AECD8FD-6096-4901-AEEF-DC9E9AE3F865}"/>
+    <hyperlink ref="I18" r:id="rId11" xr:uid="{30E523F4-0E2C-E84E-9D0D-066E220B225B}"/>
+    <hyperlink ref="I27" r:id="rId12" xr:uid="{DF01E1B8-4C36-3941-8DBE-C7B5EC78E2CC}"/>
+    <hyperlink ref="I14" r:id="rId13" xr:uid="{916D9918-7FAC-AB46-AC5F-CFFCC8216EB8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId11"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId14"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
@@ -2671,19 +2724,19 @@
           <x14:formula1>
             <xm:f>Background_info!$D$3:$D$30</xm:f>
           </x14:formula1>
-          <xm:sqref>D3:D32</xm:sqref>
+          <xm:sqref>D3:D33</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0CED9412-699B-4C7D-965B-005ACFAE9885}">
           <x14:formula1>
             <xm:f>Background_info!$C$3:$C$15</xm:f>
           </x14:formula1>
-          <xm:sqref>L3:L39</xm:sqref>
+          <xm:sqref>L3:L40</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4580CAC9-FAF7-403B-A1D9-84CB43CB97A9}">
           <x14:formula1>
             <xm:f>Background_info!$B$3:$B$7</xm:f>
           </x14:formula1>
-          <xm:sqref>H3:H32</xm:sqref>
+          <xm:sqref>H3:H33</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2694,13 +2747,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F602BA-A80C-4BEA-8ECF-F81C395286C3}">
   <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultRowHeight="14.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.75" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B1" t="str" cm="1">
         <f t="array" ref="B1:F1">TRANSPOSE(Background_info!C3:C7)</f>
         <v>pending</v>
@@ -2718,36 +2771,36 @@
         <v>rejected</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>145</v>
-      </c>
-      <c r="B2" s="36">
+        <v>144</v>
+      </c>
+      <c r="B2" s="34">
         <f>SUM(B3:B14)</f>
         <v>146.07</v>
       </c>
-      <c r="C2" s="36">
+      <c r="C2" s="34">
         <f t="shared" ref="C2:F2" si="0">SUM(C3:C14)</f>
         <v>892.29</v>
       </c>
-      <c r="D2" s="36">
+      <c r="D2" s="34">
         <f t="shared" si="0"/>
         <v>33.32</v>
       </c>
-      <c r="E2" s="36">
+      <c r="E2" s="34">
         <f t="shared" si="0"/>
         <v>87.460000000000008</v>
       </c>
-      <c r="F2" s="36">
+      <c r="F2" s="34">
         <f t="shared" si="0"/>
         <v>271.76</v>
       </c>
-      <c r="G2" s="35">
+      <c r="G2" s="33">
         <f>SUM(B2:F2)</f>
         <v>1430.8999999999999</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="str" cm="1">
         <f t="array" ref="A3:A14">Background_info!D3:D14</f>
         <v>Airframe and Structures</v>
@@ -2773,7 +2826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="str">
         <v>Propulsion</v>
       </c>
@@ -2798,7 +2851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="str">
         <v>Power</v>
       </c>
@@ -2823,7 +2876,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="str">
         <v>Flight Control and Avionics</v>
       </c>
@@ -2848,7 +2901,7 @@
         <v>28.76</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="str">
         <v>Control Surfaces and Mechanisms</v>
       </c>
@@ -2873,7 +2926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="str">
         <v>Payload and Medical Transport System</v>
       </c>
@@ -2898,7 +2951,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="str">
         <v>Communications and Ground Equipment</v>
       </c>
@@ -2923,7 +2976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="str">
         <v>Manufacturing and prototyping</v>
       </c>
@@ -2948,7 +3001,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="str">
         <v>Fasteners and Consumables</v>
       </c>
@@ -2973,7 +3026,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="str">
         <v>Testing and Safety Equipment</v>
       </c>
@@ -2998,7 +3051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="str">
         <v>Business</v>
       </c>
@@ -3023,7 +3076,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="str">
         <v>Other</v>
       </c>

</xml_diff>

<commit_message>
BOM updated with servos and wing section ESC lid holder
</commit_message>
<xml_diff>
--- a/P01/P01_06_Procurement/Table_260719_BOM.xlsx
+++ b/P01/P01_06_Procurement/Table_260719_BOM.xlsx
@@ -1,22 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25629"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\ORGOfly\ORGOfly-CAD-model\P01\P01_06_Procurement\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A1097411\Documents\GitHub\ORGOfly-CAD-Model\P01\P01_06_Procurement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D85BAC5-8216-4473-A5D4-2A725A92B518}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8420698D-8CC6-442B-B6D3-AA0254E8F595}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="1" activeTab="1" xr2:uid="{EEE73C29-3BDB-49EB-9C57-2FAD514C20AA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{EEE73C29-3BDB-49EB-9C57-2FAD514C20AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Background_info" sheetId="2" state="hidden" r:id="rId1"/>
     <sheet name="Main_Table" sheetId="1" r:id="rId2"/>
     <sheet name="Totals" sheetId="3" r:id="rId3"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Main_Table!$A$2:$N$34</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -60,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="155">
   <si>
     <t>#</t>
   </si>
@@ -227,9 +230,6 @@
     <t>HGLRC_M100_Pro</t>
   </si>
   <si>
-    <t>Servo Motor (JR connector)</t>
-  </si>
-  <si>
     <t>370 uF capacitor</t>
   </si>
   <si>
@@ -243,9 +243,6 @@
   </si>
   <si>
     <t>Power connector</t>
-  </si>
-  <si>
-    <t>Mini Servo</t>
   </si>
   <si>
     <t>Motor</t>
@@ -512,13 +509,63 @@
   </si>
   <si>
     <t>Sold in bulk. 8 pairs needed.</t>
+  </si>
+  <si>
+    <t>KingMax DCS2016SP Servo</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005012071771092.html?spm=a2g0o.productlist.main.5.1e48iOAyiOAysa&amp;algo_pvid=83ac18d0-f0b7-42c7-a0a4-143754ced9b3&amp;algo_exp_id=83ac18d0-f0b7-42c7-a0a4-143754ced9b3-4&amp;pdp_ext_f=%7B%22order%22%3A%2216%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%2120.09%2120.09%21%21%21150.60%21150.60%21%402103828617900656040581423e1064%2112000057439409399%21sea%21BG%218022761881%21ABX%211%210%21n_tag%3A-29910%3Bd%3Ab8d743bc%3Bm03_new_user%3A-29895&amp;curPageLogUid=cjkYWPn8Cvj3&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005012071771092%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Budget Servo - </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>34kg option</t>
+    </r>
+  </si>
+  <si>
+    <t>Shipping cost based on 8pcs</t>
+  </si>
+  <si>
+    <t>11-23days</t>
+  </si>
+  <si>
+    <t>KingMax S40S Servo</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">High-End Servo - </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>40kg option</t>
+    </r>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005006904005995.html?spm=a2g0o.productlist.main.1.10d0UshiUshiR3&amp;algo_pvid=c719c9d4-2227-4d7a-9ef8-5cb75879543e&amp;algo_exp_id=c719c9d4-2227-4d7a-9ef8-5cb75879543e-0&amp;pdp_ext_f=%7B%22order%22%3A%2225%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%21133.83%2186.99%21%21%211003.22%21652.10%21%4021038a8017900675691068895e0f85%2112000038669224410%21sea%21BG%218022761881%21ABX%211%210%21n_tag%3A-29910%3Bd%3Ab8d743bc%3Bm03_new_user%3A-29895&amp;curPageLogUid=lqFzD61nfosz&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005006904005995%7C_p_origin_prod%3A</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -688,7 +735,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -732,9 +779,6 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -750,9 +794,6 @@
     <xf numFmtId="16" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -765,7 +806,6 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -780,6 +820,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1180,12 +1223,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B02F099F-610B-4C2F-A80F-3888BDD56E8E}">
   <dimension ref="B2:D14"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="4" max="4" width="33.375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="33.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" ht="15">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
@@ -1196,7 +1239,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="2:4" ht="15">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
         <v>4</v>
       </c>
@@ -1207,7 +1250,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="2:4" ht="15">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
         <v>6</v>
       </c>
@@ -1218,7 +1261,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:4" ht="15">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
         <v>5</v>
       </c>
@@ -1229,7 +1272,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="2:4" ht="15">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
         <v>7</v>
       </c>
@@ -1240,9 +1283,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="2:4" ht="15">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C7" t="s">
         <v>13</v>
@@ -1251,37 +1294,37 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="2:4" ht="15">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="2:4" ht="15">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D9" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="2:4" ht="15">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="2:4" ht="15">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D11" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:4" ht="15">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="2:4" ht="15">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="2:4" ht="15">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.3">
       <c r="D14" t="s">
         <v>21</v>
       </c>
@@ -1293,33 +1336,33 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E734346-BCBC-4D9C-B399-F93315446069}">
-  <dimension ref="A1:N40"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
+  <dimension ref="A1:N41"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34.875" style="7" customWidth="1"/>
+    <col min="2" max="2" width="34.88671875" style="7" customWidth="1"/>
     <col min="3" max="3" width="50" style="2" customWidth="1"/>
-    <col min="4" max="4" width="37.625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="8.875" style="1"/>
-    <col min="7" max="7" width="8.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.125" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="12.375" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="12.375" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.875" style="1"/>
+    <col min="4" max="4" width="37.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="8.88671875" style="1"/>
+    <col min="7" max="7" width="8.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.33203125" style="1" customWidth="1"/>
+    <col min="11" max="11" width="9.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.88671875" style="1"/>
     <col min="13" max="13" width="55" style="17" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="60.625" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.875" style="2"/>
+    <col min="14" max="14" width="60.6640625" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="16384" width="8.88671875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="15">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C1" s="6"/>
       <c r="M1" s="2"/>
     </row>
-    <row r="2" spans="1:14" ht="27" customHeight="1">
+    <row r="2" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
@@ -1360,10 +1403,10 @@
         <v>14</v>
       </c>
       <c r="N2" s="11" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="15">
         <f>IF(B3&lt;&gt;"",COUNTA($B$3:B3),"")</f>
         <v>1</v>
@@ -1395,13 +1438,13 @@
       <c r="K3" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="L3" s="23" t="s">
+      <c r="L3" s="22" t="s">
         <v>36</v>
       </c>
       <c r="M3" s="16"/>
       <c r="N3" s="16"/>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A4" s="15">
         <f>IF(B4&lt;&gt;"",COUNTA($B$3:B4),"")</f>
         <v>2</v>
@@ -1437,7 +1480,7 @@
       <c r="K4" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="L4" s="23" t="s">
+      <c r="L4" s="22" t="s">
         <v>36</v>
       </c>
       <c r="M4" s="16" t="s">
@@ -1445,16 +1488,16 @@
       </c>
       <c r="N4" s="16"/>
     </row>
-    <row r="5" spans="1:14" ht="28.5">
+    <row r="5" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A5" s="15">
         <f>IF(B5&lt;&gt;"",COUNTA($B$3:B5),"")</f>
         <v>3</v>
       </c>
-      <c r="B5" s="26" t="s">
+      <c r="B5" s="24" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" s="13" t="s">
         <v>112</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>114</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>24</v>
@@ -1469,36 +1512,36 @@
         <v>1</v>
       </c>
       <c r="H5" s="15" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I5" s="8" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J5" s="15">
         <f>(G5*E5)+F5</f>
         <v>17.96</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="L5" s="23" t="s">
+        <v>115</v>
+      </c>
+      <c r="L5" s="22" t="s">
         <v>12</v>
       </c>
       <c r="M5" s="18" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="N5" s="16"/>
     </row>
-    <row r="6" spans="1:14" ht="42.75">
+    <row r="6" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A6" s="15">
         <f>IF(B6&lt;&gt;"",COUNTA($B$3:B6),"")</f>
         <v>4</v>
       </c>
-      <c r="B6" s="26" t="s">
+      <c r="B6" s="24" t="s">
         <v>40</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>24</v>
@@ -1513,32 +1556,32 @@
         <v>1</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="J6" s="15">
         <f>(G6*E6)+F6</f>
         <v>33.32</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>120</v>
-      </c>
-      <c r="L6" s="23" t="s">
-        <v>11</v>
+        <v>118</v>
+      </c>
+      <c r="L6" s="22" t="s">
+        <v>12</v>
       </c>
       <c r="M6" s="18" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="N6" s="16"/>
     </row>
-    <row r="7" spans="1:14" ht="28.5">
+    <row r="7" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A7" s="15">
         <f>IF(B7&lt;&gt;"",COUNTA($B$3:B7),"")</f>
         <v>5</v>
       </c>
-      <c r="B7" s="26" t="s">
+      <c r="B7" s="24" t="s">
         <v>37</v>
       </c>
       <c r="C7" s="13" t="s">
@@ -1550,7 +1593,7 @@
       <c r="E7" s="15">
         <v>31.22</v>
       </c>
-      <c r="F7" s="36">
+      <c r="F7" s="33">
         <v>18.75</v>
       </c>
       <c r="G7" s="15">
@@ -1560,29 +1603,29 @@
         <v>4</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="J7" s="15">
         <f t="shared" ref="J7:J23" si="0">(G7*E7)+F7</f>
         <v>143.63</v>
       </c>
-      <c r="K7" s="24" t="s">
-        <v>125</v>
-      </c>
-      <c r="L7" s="23" t="s">
+      <c r="K7" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="L7" s="22" t="s">
         <v>10</v>
       </c>
       <c r="M7" s="18" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="N7" s="16"/>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="15">
         <f>IF(B8&lt;&gt;"",COUNTA($B$3:B8),"")</f>
         <v>6</v>
       </c>
-      <c r="B8" s="26" t="s">
+      <c r="B8" s="24" t="s">
         <v>39</v>
       </c>
       <c r="C8" s="13" t="s">
@@ -1594,7 +1637,7 @@
       <c r="E8" s="15">
         <v>12.83</v>
       </c>
-      <c r="F8" s="37"/>
+      <c r="F8" s="34"/>
       <c r="G8" s="15">
         <v>2</v>
       </c>
@@ -1602,29 +1645,29 @@
         <v>4</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="J8" s="15">
         <f t="shared" si="0"/>
         <v>25.66</v>
       </c>
-      <c r="K8" s="24" t="s">
-        <v>125</v>
-      </c>
-      <c r="L8" s="23" t="s">
+      <c r="K8" s="23" t="s">
+        <v>123</v>
+      </c>
+      <c r="L8" s="22" t="s">
         <v>10</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="N8" s="16"/>
     </row>
-    <row r="9" spans="1:14" ht="28.5">
+    <row r="9" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" s="15">
         <f>IF(B9&lt;&gt;"",COUNTA($B$3:B9),"")</f>
         <v>7</v>
       </c>
-      <c r="B9" s="26" t="s">
+      <c r="B9" s="24" t="s">
         <v>47</v>
       </c>
       <c r="C9" s="13" t="s">
@@ -1646,7 +1689,7 @@
         <v>4</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="J9" s="15">
         <f t="shared" si="0"/>
@@ -1655,20 +1698,20 @@
       <c r="K9" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="L9" s="23" t="s">
+      <c r="L9" s="22" t="s">
         <v>12</v>
       </c>
       <c r="M9" s="18" t="s">
-        <v>110</v>
-      </c>
-      <c r="N9" s="31"/>
-    </row>
-    <row r="10" spans="1:14" ht="15">
+        <v>108</v>
+      </c>
+      <c r="N9" s="28"/>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="15">
         <f>IF(B10&lt;&gt;"",COUNTA($B$3:B10),"")</f>
         <v>8</v>
       </c>
-      <c r="B10" s="27" t="s">
+      <c r="B10" s="25" t="s">
         <v>50</v>
       </c>
       <c r="C10" s="13" t="s">
@@ -1690,19 +1733,19 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="L10" s="23" t="s">
+      <c r="L10" s="22" t="s">
         <v>36</v>
       </c>
       <c r="M10" s="16"/>
       <c r="N10" s="16"/>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="15">
         <f>IF(B11&lt;&gt;"",COUNTA($B$3:B11),"")</f>
         <v>9</v>
       </c>
-      <c r="B11" s="32" t="s">
-        <v>57</v>
+      <c r="B11" s="29" t="s">
+        <v>56</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>51</v>
@@ -1723,29 +1766,32 @@
         <v>4</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="J11" s="15">
         <f t="shared" si="0"/>
         <v>243</v>
       </c>
       <c r="K11" s="15" t="s">
-        <v>98</v>
-      </c>
-      <c r="L11" s="23" t="s">
+        <v>96</v>
+      </c>
+      <c r="L11" s="22" t="s">
         <v>13</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="N11" s="16" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14">
-      <c r="A12" s="15"/>
-      <c r="B12" s="28" t="s">
-        <v>145</v>
+        <v>126</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A12" s="15">
+        <f>IF(B12&lt;&gt;"",COUNTA($B$3:B12),"")</f>
+        <v>10</v>
+      </c>
+      <c r="B12" s="24" t="s">
+        <v>143</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>51</v>
@@ -1765,31 +1811,31 @@
       <c r="H12" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I12" s="35" t="s">
-        <v>144</v>
+      <c r="I12" s="32" t="s">
+        <v>142</v>
       </c>
       <c r="J12" s="15">
         <f t="shared" si="0"/>
         <v>208.57</v>
       </c>
-      <c r="K12" s="24" t="s">
-        <v>131</v>
-      </c>
-      <c r="L12" s="23" t="s">
+      <c r="K12" s="23" t="s">
+        <v>129</v>
+      </c>
+      <c r="L12" s="22" t="s">
         <v>10</v>
       </c>
       <c r="M12" s="16" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="N12" s="16"/>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A13" s="15">
-        <f>IF(B14&lt;&gt;"",COUNTA($B$3:B14),"")</f>
-        <v>12</v>
-      </c>
-      <c r="B13" s="28" t="s">
-        <v>130</v>
+        <f>IF(B13&lt;&gt;"",COUNTA($B$3:B13),"")</f>
+        <v>11</v>
+      </c>
+      <c r="B13" s="24" t="s">
+        <v>128</v>
       </c>
       <c r="C13" s="13" t="s">
         <v>51</v>
@@ -1810,35 +1856,35 @@
         <v>4</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J13" s="15">
         <f t="shared" si="0"/>
         <v>150.07</v>
       </c>
-      <c r="K13" s="24" t="s">
-        <v>131</v>
-      </c>
-      <c r="L13" s="23" t="s">
+      <c r="K13" s="23" t="s">
+        <v>129</v>
+      </c>
+      <c r="L13" s="22" t="s">
         <v>13</v>
       </c>
       <c r="M13" s="16" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="N13" s="16" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A14" s="15">
-        <f>IF(B15&lt;&gt;"",COUNTA($B$3:B15),"")</f>
-        <v>13</v>
-      </c>
-      <c r="B14" s="26" t="s">
-        <v>96</v>
+        <f>IF(B14&lt;&gt;"",COUNTA($B$3:B14),"")</f>
+        <v>12</v>
+      </c>
+      <c r="B14" s="24" t="s">
+        <v>94</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D14" s="15" t="s">
         <v>18</v>
@@ -1856,7 +1902,7 @@
         <v>4</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J14" s="15">
         <f t="shared" si="0"/>
@@ -1865,21 +1911,21 @@
       <c r="K14" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="L14" s="23" t="s">
+      <c r="L14" s="22" t="s">
         <v>10</v>
       </c>
       <c r="M14" s="16" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="N14" s="16"/>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A15" s="15">
-        <f>IF(B16&lt;&gt;"",COUNTA($B$3:B16),"")</f>
-        <v>14</v>
-      </c>
-      <c r="B15" s="32" t="s">
-        <v>56</v>
+        <f>IF(B15&lt;&gt;"",COUNTA($B$3:B15),"")</f>
+        <v>13</v>
+      </c>
+      <c r="B15" s="29" t="s">
+        <v>55</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>52</v>
@@ -1901,22 +1947,22 @@
         <v>0</v>
       </c>
       <c r="K15" s="15"/>
-      <c r="L15" s="23" t="s">
+      <c r="L15" s="22" t="s">
         <v>36</v>
       </c>
       <c r="M15" s="16"/>
       <c r="N15" s="16"/>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A16" s="15">
-        <f>IF(B17&lt;&gt;"",COUNTA($B$3:B17),"")</f>
-        <v>15</v>
+        <f>IF(B16&lt;&gt;"",COUNTA($B$3:B16),"")</f>
+        <v>14</v>
       </c>
       <c r="B16" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C16" s="13" t="s">
         <v>58</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>59</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>25</v>
@@ -1935,22 +1981,22 @@
         <v>0</v>
       </c>
       <c r="K16" s="15"/>
-      <c r="L16" s="23" t="s">
+      <c r="L16" s="22" t="s">
         <v>36</v>
       </c>
       <c r="M16" s="16"/>
       <c r="N16" s="16"/>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A17" s="15">
-        <f>IF(B18&lt;&gt;"",COUNTA($B$3:B18),"")</f>
-        <v>16</v>
-      </c>
-      <c r="B17" s="28" t="s">
+        <f>IF(B17&lt;&gt;"",COUNTA($B$3:B17),"")</f>
+        <v>15</v>
+      </c>
+      <c r="B17" s="13" t="s">
         <v>53</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>18</v>
@@ -1968,33 +2014,33 @@
         <v>4</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J17" s="15">
         <f t="shared" si="0"/>
         <v>222.3</v>
       </c>
       <c r="K17" s="15" t="s">
-        <v>93</v>
-      </c>
-      <c r="L17" s="23" t="s">
+        <v>91</v>
+      </c>
+      <c r="L17" s="22" t="s">
         <v>10</v>
       </c>
       <c r="M17" s="16" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="N17" s="16"/>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A18" s="15">
-        <f>IF(B19&lt;&gt;"",COUNTA($B$3:B19),"")</f>
-        <v>17</v>
-      </c>
-      <c r="B18" s="28" t="s">
-        <v>68</v>
+        <f>IF(B18&lt;&gt;"",COUNTA($B$3:B18),"")</f>
+        <v>16</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>66</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>25</v>
@@ -2012,33 +2058,33 @@
         <v>4</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J18" s="15">
         <f t="shared" si="0"/>
         <v>63.99</v>
       </c>
       <c r="K18" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L18" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="L18" s="22" t="s">
         <v>10</v>
       </c>
       <c r="M18" s="16" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="N18" s="16"/>
     </row>
-    <row r="19" spans="1:14">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A19" s="15">
-        <f>IF(B20&lt;&gt;"",COUNTA($B$3:B20),"")</f>
-        <v>18</v>
-      </c>
-      <c r="B19" s="26" t="s">
+        <f>IF(B19&lt;&gt;"",COUNTA($B$3:B19),"")</f>
+        <v>17</v>
+      </c>
+      <c r="B19" s="24" t="s">
         <v>54</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>25</v>
@@ -2057,22 +2103,22 @@
         <v>0</v>
       </c>
       <c r="K19" s="15"/>
-      <c r="L19" s="23" t="s">
+      <c r="L19" s="22" t="s">
         <v>36</v>
       </c>
       <c r="M19" s="16"/>
       <c r="N19" s="16"/>
     </row>
-    <row r="20" spans="1:14" ht="28.5">
+    <row r="20" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A20" s="15">
-        <f>IF(B21&lt;&gt;"",COUNTA($B$3:B21),"")</f>
-        <v>19</v>
-      </c>
-      <c r="B20" s="28" t="s">
-        <v>74</v>
+        <f>IF(B20&lt;&gt;"",COUNTA($B$3:B20),"")</f>
+        <v>18</v>
+      </c>
+      <c r="B20" s="24" t="s">
+        <v>72</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>30</v>
@@ -2090,33 +2136,33 @@
         <v>4</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J20" s="15">
         <f t="shared" si="0"/>
         <v>17.79</v>
       </c>
       <c r="K20" s="15" t="s">
-        <v>136</v>
-      </c>
-      <c r="L20" s="23" t="s">
+        <v>134</v>
+      </c>
+      <c r="L20" s="22" t="s">
         <v>10</v>
       </c>
       <c r="M20" s="16" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="N20" s="16"/>
     </row>
-    <row r="21" spans="1:14" ht="28.5">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="15">
-        <f>IF(B22&lt;&gt;"",COUNTA($B$3:B22),"")</f>
-        <v>20</v>
-      </c>
-      <c r="B21" s="26" t="s">
-        <v>76</v>
+        <f>IF(B21&lt;&gt;"",COUNTA($B$3:B21),"")</f>
+        <v>19</v>
+      </c>
+      <c r="B21" s="24" t="s">
+        <v>74</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>30</v>
@@ -2134,7 +2180,7 @@
         <v>4</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="J21" s="15">
         <f t="shared" si="0"/>
@@ -2143,24 +2189,24 @@
       <c r="K21" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="L21" s="23" t="s">
+      <c r="L21" s="22" t="s">
         <v>36</v>
       </c>
       <c r="M21" s="16" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="N21" s="16"/>
     </row>
-    <row r="22" spans="1:14">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A22" s="15">
-        <f>IF(B23&lt;&gt;"",COUNTA($B$3:B23),"")</f>
-        <v>21</v>
-      </c>
-      <c r="B22" s="26" t="s">
-        <v>78</v>
+        <f>IF(B22&lt;&gt;"",COUNTA($B$3:B22),"")</f>
+        <v>20</v>
+      </c>
+      <c r="B22" s="24" t="s">
+        <v>76</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D22" s="15" t="s">
         <v>30</v>
@@ -2178,7 +2224,7 @@
         <v>4</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="J22" s="15">
         <f t="shared" si="0"/>
@@ -2187,24 +2233,24 @@
       <c r="K22" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="L22" s="23" t="s">
+      <c r="L22" s="22" t="s">
         <v>36</v>
       </c>
       <c r="M22" s="16" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="N22" s="16"/>
     </row>
-    <row r="23" spans="1:14">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A23" s="15">
-        <f>IF(B24&lt;&gt;"",COUNTA($B$3:B24),"")</f>
-        <v>22</v>
-      </c>
-      <c r="B23" s="26" t="s">
-        <v>86</v>
+        <f>IF(B23&lt;&gt;"",COUNTA($B$3:B23),"")</f>
+        <v>21</v>
+      </c>
+      <c r="B23" s="24" t="s">
+        <v>84</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="D23" s="15" t="s">
         <v>30</v>
@@ -2222,7 +2268,7 @@
         <v>4</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="J23" s="15">
         <f t="shared" si="0"/>
@@ -2231,344 +2277,358 @@
       <c r="K23" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="L23" s="23" t="s">
+      <c r="L23" s="22" t="s">
         <v>36</v>
       </c>
       <c r="M23" s="16" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="N23" s="16"/>
     </row>
-    <row r="24" spans="1:14" ht="12.75" customHeight="1">
+    <row r="24" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="15">
+        <f>IF(B24&lt;&gt;"",COUNTA($B$3:B24),"")</f>
+        <v>22</v>
+      </c>
+      <c r="B24" s="27" t="s">
+        <v>78</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="D24" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="E24" s="15">
+        <v>8.66</v>
+      </c>
+      <c r="F24" s="15">
+        <v>0</v>
+      </c>
+      <c r="G24" s="15">
+        <v>1</v>
+      </c>
+      <c r="H24" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I24" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="J24" s="15">
+        <f t="shared" ref="J24:J30" si="1">(G24*E24)+F24</f>
+        <v>8.66</v>
+      </c>
+      <c r="K24" s="15" t="s">
+        <v>48</v>
+      </c>
+      <c r="L24" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M24" s="16"/>
+      <c r="N24" s="16"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A25" s="15">
         <f>IF(B25&lt;&gt;"",COUNTA($B$3:B25),"")</f>
         <v>23</v>
       </c>
-      <c r="B24" s="29" t="s">
-        <v>80</v>
-      </c>
-      <c r="C24" s="13" t="s">
-        <v>81</v>
-      </c>
-      <c r="D24" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="E24" s="15">
-        <v>8.66</v>
-      </c>
-      <c r="F24" s="15">
-        <v>0</v>
-      </c>
-      <c r="G24" s="15">
-        <v>1</v>
-      </c>
-      <c r="H24" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="I24" s="13" t="s">
-        <v>79</v>
-      </c>
-      <c r="J24" s="15">
-        <f t="shared" ref="J24:J29" si="1">(G24*E24)+F24</f>
-        <v>8.66</v>
-      </c>
-      <c r="K24" s="15" t="s">
-        <v>48</v>
-      </c>
-      <c r="L24" s="23" t="s">
+      <c r="B25" s="35" t="s">
+        <v>147</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="D25" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E25" s="15">
+        <v>20.09</v>
+      </c>
+      <c r="F25" s="15">
+        <v>15.25</v>
+      </c>
+      <c r="G25" s="15">
+        <v>8</v>
+      </c>
+      <c r="H25" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I25" s="3" t="s">
+        <v>148</v>
+      </c>
+      <c r="J25" s="15">
+        <f t="shared" si="1"/>
+        <v>175.97</v>
+      </c>
+      <c r="K25" s="15" t="s">
+        <v>151</v>
+      </c>
+      <c r="L25" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="M24" s="16"/>
-      <c r="N24" s="16"/>
-    </row>
-    <row r="25" spans="1:14" ht="15">
-      <c r="A25" s="15">
+      <c r="M25" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="N25" s="16"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A26" s="15">
         <f>IF(B26&lt;&gt;"",COUNTA($B$3:B26),"")</f>
         <v>24</v>
       </c>
-      <c r="B25" s="19" t="s">
-        <v>61</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="D25" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="E25" s="15"/>
-      <c r="F25" s="15"/>
-      <c r="G25" s="15">
-        <v>4</v>
-      </c>
-      <c r="H25" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="I25" s="3"/>
-      <c r="J25" s="15">
+      <c r="B26" s="35" t="s">
+        <v>152</v>
+      </c>
+      <c r="C26" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="D26" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E26" s="15">
+        <v>86.99</v>
+      </c>
+      <c r="F26" s="15">
+        <v>2.17</v>
+      </c>
+      <c r="G26" s="15">
+        <v>8</v>
+      </c>
+      <c r="H26" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I26" s="3" t="s">
+        <v>154</v>
+      </c>
+      <c r="J26" s="15">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="K25" s="15"/>
-      <c r="L25" s="23" t="s">
+        <v>698.08999999999992</v>
+      </c>
+      <c r="K26" s="15" t="s">
+        <v>118</v>
+      </c>
+      <c r="L26" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="M25" s="16"/>
-      <c r="N25" s="16"/>
-    </row>
-    <row r="26" spans="1:14" ht="28.5">
-      <c r="A26" s="15">
+      <c r="M26" s="16" t="s">
+        <v>150</v>
+      </c>
+      <c r="N26" s="16"/>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A27" s="15">
         <f>IF(B27&lt;&gt;"",COUNTA($B$3:B27),"")</f>
         <v>25</v>
       </c>
-      <c r="B26" s="25" t="s">
-        <v>88</v>
-      </c>
-      <c r="C26" s="13" t="s">
-        <v>62</v>
-      </c>
-      <c r="D26" s="15" t="s">
+      <c r="B27" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="D27" s="15" t="s">
         <v>18</v>
       </c>
-      <c r="E26" s="15">
+      <c r="E27" s="15">
         <v>174.99</v>
       </c>
-      <c r="F26" s="15">
-        <v>0</v>
-      </c>
-      <c r="G26" s="15">
+      <c r="F27" s="15">
+        <v>0</v>
+      </c>
+      <c r="G27" s="15">
         <v>1</v>
       </c>
-      <c r="H26" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="I26" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="J26" s="15">
+      <c r="H27" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I27" s="8" t="s">
+        <v>85</v>
+      </c>
+      <c r="J27" s="15">
         <f t="shared" si="1"/>
         <v>174.99</v>
       </c>
-      <c r="K26" s="15" t="s">
-        <v>89</v>
-      </c>
-      <c r="L26" s="23" t="s">
+      <c r="K27" s="15" t="s">
+        <v>87</v>
+      </c>
+      <c r="L27" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="M26" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="N26" s="16"/>
-    </row>
-    <row r="27" spans="1:14">
-      <c r="A27" s="15">
+      <c r="M27" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="N27" s="16"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A28" s="15">
         <f>IF(B28&lt;&gt;"",COUNTA($B$3:B28),"")</f>
         <v>26</v>
       </c>
-      <c r="B27" s="30" t="s">
-        <v>65</v>
-      </c>
-      <c r="C27" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="D27" s="15" t="s">
+      <c r="B28" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="D28" s="15" t="s">
         <v>19</v>
       </c>
-      <c r="E27" s="15">
+      <c r="E28" s="15">
         <v>31.9</v>
       </c>
-      <c r="F27" s="15">
+      <c r="F28" s="15">
         <v>8.4700000000000006</v>
       </c>
-      <c r="G27" s="15">
+      <c r="G28" s="15">
         <v>1</v>
       </c>
-      <c r="H27" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="I27" s="8" t="s">
-        <v>139</v>
-      </c>
-      <c r="J27" s="15">
+      <c r="H28" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I28" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
         <v>40.369999999999997</v>
       </c>
-      <c r="K27" s="15" t="s">
+      <c r="K28" s="15" t="s">
+        <v>136</v>
+      </c>
+      <c r="L28" s="22" t="s">
+        <v>10</v>
+      </c>
+      <c r="M28" s="16" t="s">
         <v>138</v>
       </c>
-      <c r="L27" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="M27" s="16" t="s">
-        <v>140</v>
-      </c>
-      <c r="N27" s="16"/>
-    </row>
-    <row r="28" spans="1:14">
-      <c r="A28" s="15">
+      <c r="N28" s="16"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A29" s="15">
         <f>IF(B29&lt;&gt;"",COUNTA($B$3:B29),"")</f>
         <v>27</v>
       </c>
-      <c r="B28" s="25" t="s">
-        <v>63</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>146</v>
-      </c>
-      <c r="D28" s="15" t="s">
+      <c r="B29" s="13" t="s">
+        <v>61</v>
+      </c>
+      <c r="C29" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="D29" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="E28" s="15">
+      <c r="E29" s="15">
         <v>53.49</v>
       </c>
-      <c r="F28" s="15">
-        <v>0</v>
-      </c>
-      <c r="G28" s="15">
+      <c r="F29" s="15">
+        <v>0</v>
+      </c>
+      <c r="G29" s="15">
         <v>1</v>
       </c>
-      <c r="H28" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="I28" s="8" t="s">
-        <v>141</v>
-      </c>
-      <c r="J28" s="15">
+      <c r="H29" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I29" s="8" t="s">
+        <v>139</v>
+      </c>
+      <c r="J29" s="15">
         <f t="shared" si="1"/>
         <v>53.49</v>
       </c>
-      <c r="K28" s="15" t="s">
-        <v>91</v>
-      </c>
-      <c r="L28" s="23" t="s">
+      <c r="K29" s="15" t="s">
+        <v>89</v>
+      </c>
+      <c r="L29" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="M28" s="16" t="s">
-        <v>142</v>
-      </c>
-      <c r="N28" s="16"/>
-    </row>
-    <row r="29" spans="1:14" ht="28.5">
-      <c r="A29" s="15">
+      <c r="M29" s="16" t="s">
+        <v>140</v>
+      </c>
+      <c r="N29" s="16"/>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A30" s="15">
         <f>IF(B30&lt;&gt;"",COUNTA($B$3:B30),"")</f>
         <v>28</v>
       </c>
-      <c r="B29" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="C29" s="13" t="s">
-        <v>71</v>
-      </c>
-      <c r="D29" s="15" t="s">
+      <c r="B30" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="C30" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="D30" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E29" s="15"/>
-      <c r="F29" s="15"/>
-      <c r="G29" s="15">
+      <c r="E30" s="15"/>
+      <c r="F30" s="15"/>
+      <c r="G30" s="15">
         <v>1</v>
       </c>
-      <c r="H29" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="I29" s="3"/>
-      <c r="J29" s="15">
+      <c r="H30" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I30" s="3"/>
+      <c r="J30" s="15">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="K29" s="15"/>
-      <c r="L29" s="23" t="s">
+      <c r="K30" s="15"/>
+      <c r="L30" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="M29" s="16"/>
-      <c r="N29" s="16"/>
-    </row>
-    <row r="30" spans="1:14" ht="28.5">
-      <c r="A30" s="15">
+      <c r="M30" s="16"/>
+      <c r="N30" s="16"/>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A31" s="15">
         <f>IF(B31&lt;&gt;"",COUNTA($B$3:B31),"")</f>
         <v>29</v>
       </c>
-      <c r="B30" s="20" t="s">
-        <v>104</v>
-      </c>
-      <c r="C30" s="20" t="s">
-        <v>99</v>
-      </c>
-      <c r="D30" s="15" t="s">
+      <c r="B31" s="19" t="s">
+        <v>102</v>
+      </c>
+      <c r="C31" s="19" t="s">
+        <v>97</v>
+      </c>
+      <c r="D31" s="15" t="s">
         <v>25</v>
       </c>
-      <c r="E30" s="22">
+      <c r="E31" s="21">
         <v>6.99</v>
       </c>
-      <c r="F30" s="15"/>
-      <c r="G30" s="15">
-        <v>4</v>
-      </c>
-      <c r="H30" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="I30" s="21" t="s">
-        <v>102</v>
-      </c>
-      <c r="J30" s="15">
-        <f t="shared" ref="J30" si="2">(G30*E30)+F30</f>
+      <c r="F31" s="15"/>
+      <c r="G31" s="15">
+        <v>4</v>
+      </c>
+      <c r="H31" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I31" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="J31" s="15">
+        <f t="shared" ref="J31" si="2">(G31*E31)+F31</f>
         <v>27.96</v>
       </c>
-      <c r="K30" s="15"/>
-      <c r="L30" s="23" t="s">
+      <c r="K31" s="15"/>
+      <c r="L31" s="22" t="s">
         <v>36</v>
       </c>
-      <c r="M30" s="16"/>
-      <c r="N30" s="16"/>
-    </row>
-    <row r="31" spans="1:14">
-      <c r="A31" s="15">
+      <c r="M31" s="16"/>
+      <c r="N31" s="16"/>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A32" s="15">
         <f>IF(B32&lt;&gt;"",COUNTA($B$3:B32),"")</f>
         <v>30</v>
       </c>
-      <c r="B31" s="20" t="s">
-        <v>103</v>
-      </c>
-      <c r="C31" s="20" t="s">
-        <v>100</v>
-      </c>
-      <c r="D31" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="E31" s="15">
-        <v>7.19</v>
-      </c>
-      <c r="F31" s="15"/>
-      <c r="G31" s="15">
-        <v>2</v>
-      </c>
-      <c r="H31" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="I31" s="21" t="s">
+      <c r="B32" s="19" t="s">
         <v>101</v>
       </c>
-      <c r="J31" s="15">
-        <f t="shared" ref="J31" si="3">(G31*E31)+F31</f>
-        <v>14.38</v>
-      </c>
-      <c r="K31" s="15"/>
-      <c r="L31" s="23" t="s">
-        <v>13</v>
-      </c>
-      <c r="M31" s="16"/>
-      <c r="N31" s="16" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="32" spans="1:14">
-      <c r="A32" s="15">
-        <f>IF(B33&lt;&gt;"",COUNTA($B$3:B33),"")</f>
-        <v>31</v>
-      </c>
-      <c r="B32" s="20" t="s">
-        <v>105</v>
-      </c>
-      <c r="C32" s="20" t="s">
-        <v>100</v>
+      <c r="C32" s="19" t="s">
+        <v>98</v>
       </c>
       <c r="D32" s="15" t="s">
         <v>25</v>
@@ -2583,86 +2643,136 @@
       <c r="H32" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I32" s="21" t="s">
-        <v>101</v>
+      <c r="I32" s="20" t="s">
+        <v>99</v>
       </c>
       <c r="J32" s="15">
-        <f t="shared" ref="J32" si="4">(G32*E32)+F32</f>
+        <f t="shared" ref="J32" si="3">(G32*E32)+F32</f>
         <v>14.38</v>
       </c>
       <c r="K32" s="15"/>
-      <c r="L32" s="23" t="s">
+      <c r="L32" s="22" t="s">
         <v>13</v>
       </c>
       <c r="M32" s="16"/>
       <c r="N32" s="16" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="33" spans="1:14">
-      <c r="A33" s="2">
-        <v>30</v>
-      </c>
-      <c r="B33" s="20" t="s">
-        <v>107</v>
-      </c>
-      <c r="C33" s="20" t="s">
-        <v>108</v>
+        <v>125</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A33" s="15">
+        <f>IF(B33&lt;&gt;"",COUNTA($B$3:B33),"")</f>
+        <v>31</v>
+      </c>
+      <c r="B33" s="19" t="s">
+        <v>103</v>
+      </c>
+      <c r="C33" s="19" t="s">
+        <v>98</v>
       </c>
       <c r="D33" s="15" t="s">
         <v>25</v>
       </c>
       <c r="E33" s="15">
-        <v>4.8899999999999997</v>
+        <v>7.19</v>
       </c>
       <c r="F33" s="15"/>
       <c r="G33" s="15">
+        <v>2</v>
+      </c>
+      <c r="H33" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I33" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="J33" s="15">
+        <f t="shared" ref="J33" si="4">(G33*E33)+F33</f>
+        <v>14.38</v>
+      </c>
+      <c r="K33" s="15"/>
+      <c r="L33" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="M33" s="16"/>
+      <c r="N33" s="16" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A34" s="15">
+        <f>IF(B34&lt;&gt;"",COUNTA($B$3:B34),"")</f>
+        <v>32</v>
+      </c>
+      <c r="B34" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="C34" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="D34" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="E34" s="15">
+        <v>4.8899999999999997</v>
+      </c>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15">
         <v>1</v>
       </c>
-      <c r="H33" s="15" t="s">
-        <v>4</v>
-      </c>
-      <c r="I33" s="21" t="s">
-        <v>106</v>
-      </c>
-      <c r="J33" s="15">
-        <f t="shared" ref="J33" si="5">(G33*E33)+F33</f>
+      <c r="H34" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I34" s="20" t="s">
+        <v>104</v>
+      </c>
+      <c r="J34" s="15">
+        <f t="shared" ref="J34" si="5">(G34*E34)+F34</f>
         <v>4.8899999999999997</v>
       </c>
-      <c r="K33" s="15"/>
-      <c r="L33" s="23" t="s">
+      <c r="K34" s="15"/>
+      <c r="L34" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="M33" s="16"/>
-      <c r="N33" s="16"/>
-    </row>
-    <row r="34" spans="1:14">
-      <c r="L34" s="23"/>
-    </row>
-    <row r="35" spans="1:14">
-      <c r="L35" s="23"/>
-    </row>
-    <row r="36" spans="1:14">
-      <c r="L36" s="23"/>
-    </row>
-    <row r="37" spans="1:14">
-      <c r="L37" s="23"/>
-    </row>
-    <row r="38" spans="1:14">
-      <c r="L38" s="23"/>
-    </row>
-    <row r="39" spans="1:14">
-      <c r="L39" s="23"/>
-    </row>
-    <row r="40" spans="1:14">
-      <c r="L40" s="23"/>
+      <c r="M34" s="16"/>
+      <c r="N34" s="16"/>
+    </row>
+    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A35" s="15" t="str">
+        <f>IF(B35&lt;&gt;"",COUNTA($B$3:B35),"")</f>
+        <v/>
+      </c>
+      <c r="L35" s="22"/>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="A36" s="15" t="str">
+        <f>IF(B36&lt;&gt;"",COUNTA($B$3:B36),"")</f>
+        <v/>
+      </c>
+      <c r="L36" s="22"/>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="L37" s="22"/>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="L38" s="22"/>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="L39" s="22"/>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="L40" s="22"/>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="L41" s="22"/>
     </row>
   </sheetData>
+  <autoFilter ref="A2:N34" xr:uid="{0E734346-BCBC-4D9C-B399-F93315446069}"/>
   <mergeCells count="1">
     <mergeCell ref="F7:F8"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
-  <conditionalFormatting sqref="L3:L6 L15:L40 L10:L12">
+  <conditionalFormatting sqref="L3:L6 L10:L12 L28:L41 L15:L26">
     <cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="pending">
       <formula>NOT(ISERROR(SEARCH("pending",L3)))</formula>
     </cfRule>
@@ -2670,7 +2780,7 @@
       <formula>$B2="approved"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L3:L40">
+  <conditionalFormatting sqref="L3:L41">
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="approved">
       <formula>NOT(ISERROR(SEARCH("approved",L3)))</formula>
     </cfRule>
@@ -2684,7 +2794,7 @@
       <formula>NOT(ISERROR(SEARCH("received",L3)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L40">
+  <conditionalFormatting sqref="L4:L41">
     <cfRule type="expression" priority="9">
       <formula>#REF!="approved"</formula>
     </cfRule>
@@ -2704,20 +2814,27 @@
       <formula>$B5="approved"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="L12:L13">
+    <cfRule type="expression" priority="27">
+      <formula>$B10="approved"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L12:L14">
+    <cfRule type="containsText" dxfId="1" priority="22" operator="containsText" text="pending">
+      <formula>NOT(ISERROR(SEARCH("pending",L12)))</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L14">
-    <cfRule type="containsText" dxfId="1" priority="22" operator="containsText" text="pending">
-      <formula>NOT(ISERROR(SEARCH("pending",L14)))</formula>
-    </cfRule>
     <cfRule type="expression" priority="23">
       <formula>$B11="approved"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L12:L13">
-    <cfRule type="containsText" dxfId="0" priority="26" operator="containsText" text="pending">
-      <formula>NOT(ISERROR(SEARCH("pending",L12)))</formula>
+  <conditionalFormatting sqref="L27">
+    <cfRule type="containsText" dxfId="0" priority="30" operator="containsText" text="pending">
+      <formula>NOT(ISERROR(SEARCH("pending",L27)))</formula>
     </cfRule>
-    <cfRule type="expression" priority="27">
-      <formula>$B10="approved"</formula>
+    <cfRule type="expression" priority="31">
+      <formula>$B25="approved"</formula>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
@@ -2726,13 +2843,13 @@
     <hyperlink ref="I6" r:id="rId3" xr:uid="{3002E511-E2F5-4C78-B094-E6DD7CF3B671}"/>
     <hyperlink ref="I7" r:id="rId4" xr:uid="{46C8B073-4590-4C63-B6E5-2A03FB1E94E6}"/>
     <hyperlink ref="I8" r:id="rId5" xr:uid="{7085C41A-4F68-4A70-A26C-EBBC546A59EE}"/>
-    <hyperlink ref="I26" r:id="rId6" xr:uid="{AC3997AD-8B71-448A-BCF4-2A0239242A9A}"/>
+    <hyperlink ref="I27" r:id="rId6" xr:uid="{AC3997AD-8B71-448A-BCF4-2A0239242A9A}"/>
     <hyperlink ref="I20" r:id="rId7" display="https://www.aliexpress.com/item/1005003122596249.html?spm=a2g0o.productlist.main.23.70394477bJf9UQ&amp;algo_pvid=169d2b7f-426b-4582-b7f2-1a69c234abe7&amp;algo_exp_id=169d2b7f-426b-4582-b7f2-1a69c234abe7-20&amp;pdp_ext_f=%7B%22order%22%3A%222145%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%217.69%215.92%21%21%218.62%216.64%21%400b8848e317897611280765333e0f49%2112000024217621966%21sea%21BG%210%21ABX%211%210%21n_tag%3A-29910%3Bd%3Abb4150ed%3Bm03_new_user%3A-29895%3BpisId%3A5000000217831009&amp;curPageLogUid=7PGL6jiPmM9H&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005003122596249%7C_p_origin_prod%3A" xr:uid="{93C2ADC8-BF07-46BD-B25F-9FBD4C8B46B2}"/>
     <hyperlink ref="I17" r:id="rId8" xr:uid="{1F742A85-6E5F-4512-8BB8-6CC598E9162E}"/>
     <hyperlink ref="I13" r:id="rId9" xr:uid="{B0912176-1BFC-47C4-867E-D85D256F8603}"/>
-    <hyperlink ref="I28" r:id="rId10" xr:uid="{3AECD8FD-6096-4901-AEEF-DC9E9AE3F865}"/>
+    <hyperlink ref="I29" r:id="rId10" xr:uid="{3AECD8FD-6096-4901-AEEF-DC9E9AE3F865}"/>
     <hyperlink ref="I18" r:id="rId11" xr:uid="{30E523F4-0E2C-E84E-9D0D-066E220B225B}"/>
-    <hyperlink ref="I27" r:id="rId12" xr:uid="{DF01E1B8-4C36-3941-8DBE-C7B5EC78E2CC}"/>
+    <hyperlink ref="I28" r:id="rId12" xr:uid="{DF01E1B8-4C36-3941-8DBE-C7B5EC78E2CC}"/>
     <hyperlink ref="I14" r:id="rId13" xr:uid="{916D9918-7FAC-AB46-AC5F-CFFCC8216EB8}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2744,19 +2861,19 @@
           <x14:formula1>
             <xm:f>Background_info!$D$3:$D$30</xm:f>
           </x14:formula1>
-          <xm:sqref>D3:D33</xm:sqref>
+          <xm:sqref>D3:D34</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0CED9412-699B-4C7D-965B-005ACFAE9885}">
           <x14:formula1>
             <xm:f>Background_info!$C$3:$C$15</xm:f>
           </x14:formula1>
-          <xm:sqref>L3:L40</xm:sqref>
+          <xm:sqref>L3:L41</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4580CAC9-FAF7-403B-A1D9-84CB43CB97A9}">
           <x14:formula1>
             <xm:f>Background_info!$B$3:$B$7</xm:f>
           </x14:formula1>
-          <xm:sqref>H3:H33</xm:sqref>
+          <xm:sqref>H3:H34</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2767,13 +2884,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F602BA-A80C-4BEA-8ECF-F81C395286C3}">
   <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="33" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="B1" t="str" cm="1">
         <f t="array" ref="B1:F1">TRANSPOSE(Background_info!C3:C7)</f>
         <v>pending</v>
@@ -2791,36 +2908,36 @@
         <v>rejected</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>143</v>
-      </c>
-      <c r="B2" s="34">
+        <v>141</v>
+      </c>
+      <c r="B2" s="31">
         <f>SUM(B3:B14)</f>
-        <v>108.28</v>
-      </c>
-      <c r="C2" s="34">
+        <v>982.34</v>
+      </c>
+      <c r="C2" s="31">
         <f t="shared" ref="C2:F2" si="0">SUM(C3:C14)</f>
         <v>988.58</v>
       </c>
-      <c r="D2" s="34">
+      <c r="D2" s="31">
         <f t="shared" si="0"/>
-        <v>33.32</v>
-      </c>
-      <c r="E2" s="34">
+        <v>0</v>
+      </c>
+      <c r="E2" s="31">
         <f t="shared" si="0"/>
-        <v>87.460000000000008</v>
-      </c>
-      <c r="F2" s="34">
+        <v>120.78</v>
+      </c>
+      <c r="F2" s="31">
         <f t="shared" si="0"/>
         <v>421.83</v>
       </c>
-      <c r="G2" s="33">
+      <c r="G2" s="30">
         <f>SUM(B2:F2)</f>
-        <v>1639.47</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7">
+        <v>2513.5300000000002</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="str" cm="1">
         <f t="array" ref="A3:A14">Background_info!D3:D14</f>
         <v>Airframe and Structures</v>
@@ -2835,18 +2952,18 @@
       </c>
       <c r="D3">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A3,Main_Table!$L:$L,D$1)</f>
-        <v>33.32</v>
+        <v>0</v>
       </c>
       <c r="E3">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A3,Main_Table!$L:$L,E$1)</f>
-        <v>17.96</v>
+        <v>51.28</v>
       </c>
       <c r="F3">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A3,Main_Table!$L:$L,F$1)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="str">
         <v>Propulsion</v>
       </c>
@@ -2871,7 +2988,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="str">
         <v>Power</v>
       </c>
@@ -2896,13 +3013,13 @@
         <v>393.07</v>
       </c>
     </row>
-    <row r="6" spans="1:7">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="str">
         <v>Flight Control and Avionics</v>
       </c>
       <c r="B6">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A6,Main_Table!$L:$L,B$1)</f>
-        <v>27.96</v>
+        <v>902.02</v>
       </c>
       <c r="C6">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A6,Main_Table!$L:$L,C$1)</f>
@@ -2921,7 +3038,7 @@
         <v>28.76</v>
       </c>
     </row>
-    <row r="7" spans="1:7">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="str">
         <v>Control Surfaces and Mechanisms</v>
       </c>
@@ -2946,7 +3063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="str">
         <v>Payload and Medical Transport System</v>
       </c>
@@ -2971,7 +3088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" t="str">
         <v>Communications and Ground Equipment</v>
       </c>
@@ -2996,7 +3113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="str">
         <v>Manufacturing and prototyping</v>
       </c>
@@ -3021,7 +3138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" t="str">
         <v>Fasteners and Consumables</v>
       </c>
@@ -3046,7 +3163,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" t="str">
         <v>Testing and Safety Equipment</v>
       </c>
@@ -3071,7 +3188,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" t="str">
         <v>Business</v>
       </c>
@@ -3096,7 +3213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="str">
         <v>Other</v>
       </c>

</xml_diff>

<commit_message>
BOM update + invoices
09/10/26
</commit_message>
<xml_diff>
--- a/P01/P01_06_Procurement/Table_260719_BOM.xlsx
+++ b/P01/P01_06_Procurement/Table_260719_BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11004"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\A1097411\Documents\GitHub\ORGOfly-CAD-Model\P01\P01_06_Procurement\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/martin/Documents/GitHub/ORGOfly-CAD-model/P01/P01_06_Procurement/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11B6D685-B33B-4B8E-A691-8CE490673242}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D03643A1-2488-4844-9E6C-7FA7918467C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" firstSheet="1" activeTab="1" xr2:uid="{EEE73C29-3BDB-49EB-9C57-2FAD514C20AA}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17740" activeTab="1" xr2:uid="{EEE73C29-3BDB-49EB-9C57-2FAD514C20AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Background_info" sheetId="2" state="hidden" r:id="rId1"/>
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="171">
   <si>
     <t>#</t>
   </si>
@@ -225,9 +225,6 @@
   </si>
   <si>
     <t>SQESC_12100</t>
-  </si>
-  <si>
-    <t>HGLRC_M100_Pro</t>
   </si>
   <si>
     <t>370 uF capacitor</t>
@@ -500,9 +497,6 @@
   </si>
   <si>
     <t>Ovonic Roam 6S 8Ah 150C</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> </t>
   </si>
   <si>
     <t>Lower density option available</t>
@@ -559,6 +553,60 @@
   </si>
   <si>
     <t>https://www.aliexpress.com/item/1005006904005995.html?spm=a2g0o.productlist.main.1.10d0UshiUshiR3&amp;algo_pvid=c719c9d4-2227-4d7a-9ef8-5cb75879543e&amp;algo_exp_id=c719c9d4-2227-4d7a-9ef8-5cb75879543e-0&amp;pdp_ext_f=%7B%22order%22%3A%2225%22%2C%22eval%22%3A%221%22%2C%22fromPage%22%3A%22search%22%7D&amp;pdp_npi=6%40dis%21EUR%21133.83%2186.99%21%21%211003.22%21652.10%21%4021038a8017900675691068895e0f85%2112000038669224410%21sea%21BG%218022761881%21ABX%211%210%21n_tag%3A-29910%3Bd%3Ab8d743bc%3Bm03_new_user%3A-29895&amp;curPageLogUid=lqFzD61nfosz&amp;utparam-url=scene%3Asearch%7Cquery_from%3A%7Cx_object_id%3A1005006904005995%7C_p_origin_prod%3A</t>
+  </si>
+  <si>
+    <t>Radiomaster TX16s MK3 + XR4 Reciever</t>
+  </si>
+  <si>
+    <t>Ovonic Roam 6S 6Ah5 150C XT90-S</t>
+  </si>
+  <si>
+    <t>better density, cheaper per W, ability to swap 2 packs in tests</t>
+  </si>
+  <si>
+    <t>transmitter + reciever (seller confirmed LBT - EU standard)</t>
+  </si>
+  <si>
+    <t>https://www.ebay.co.uk/itm/278435436885</t>
+  </si>
+  <si>
+    <t>https://www.ampow.com/products/ovonic-roam-series-6s-lipo-battery-6500mah-6s1p-150c-22-2v-long-range-lipo-battery-with-xt90-s-anti-spark-plug-for-x8-cinelifte-long-range-multirotor-x-class?variant=46118867075316</t>
+  </si>
+  <si>
+    <t>RadioMaster 5000mAh 2S 7.4V Li-ion Battery</t>
+  </si>
+  <si>
+    <t>best option for main battery for transmitter (sold separately)</t>
+  </si>
+  <si>
+    <t>https://motionrc.com/eu/products/radiomaster-5000mah-2s-7-4v-li-ion-battery-with-xt30-connector-hp0157-batt-5a2s?utm_source=Abandoned+Checkout+(3+Emails)+-+Odoo&amp;utm_medium=email&amp;utm_campaign=Abandoned+Checkout:+Email+1+(Rfc2Th)&amp;_kx=X52hvKiu13nlLG7L3s0Wp1W1Q7QTzfEVi-kaGTYW3IGFDRwXBr78uVpHw36A19cw.HGcQyL</t>
+  </si>
+  <si>
+    <t>7-10 days</t>
+  </si>
+  <si>
+    <t>Holybro Micro M10 GPS With IST8310 Digital Compass Ceramic Patch Antenna</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005008932272456.html?spm=a2g0o.order_list.order_list_main.22.1d391802SsgA9y</t>
+  </si>
+  <si>
+    <t>Transmitter battery</t>
+  </si>
+  <si>
+    <t>Not compatible with the newly selected transmitter</t>
+  </si>
+  <si>
+    <t>saved for next iterations, not needed for prototype phase</t>
+  </si>
+  <si>
+    <t>TBS Crossfire Diversity Nano RX Receiver FPV Long Range</t>
+  </si>
+  <si>
+    <t>XR4 dual band reciever planned</t>
+  </si>
+  <si>
+    <t>Тransmitter + reciever</t>
   </si>
 </sst>
 </file>
@@ -1211,12 +1259,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B02F099F-610B-4C2F-A80F-3888BDD56E8E}">
   <dimension ref="B2:D14"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="4" max="4" width="33.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
@@ -1227,7 +1275,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B3" t="s">
         <v>4</v>
       </c>
@@ -1238,7 +1286,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B4" t="s">
         <v>6</v>
       </c>
@@ -1249,7 +1297,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="5" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B5" t="s">
         <v>5</v>
       </c>
@@ -1260,7 +1308,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B6" t="s">
         <v>7</v>
       </c>
@@ -1271,9 +1319,9 @@
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:4" x14ac:dyDescent="0.2">
       <c r="B7" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C7" t="s">
         <v>13</v>
@@ -1282,37 +1330,37 @@
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D8" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="9" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D9" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="10" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D10" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D11" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="12" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D13" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="2:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:4" x14ac:dyDescent="0.2">
       <c r="D14" t="s">
         <v>21</v>
       </c>
@@ -1325,32 +1373,32 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0E734346-BCBC-4D9C-B399-F93315446069}">
   <dimension ref="A1:N41"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="3" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="34.88671875" style="7" customWidth="1"/>
+    <col min="2" max="2" width="34.83203125" style="7" customWidth="1"/>
     <col min="3" max="3" width="50" style="2" customWidth="1"/>
     <col min="4" max="4" width="37.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="8.88671875" style="1"/>
-    <col min="7" max="7" width="8.109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="8.83203125" style="1"/>
+    <col min="7" max="7" width="8.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="5.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="12.33203125" style="1" customWidth="1"/>
-    <col min="11" max="11" width="9.44140625" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.88671875" style="1"/>
+    <col min="11" max="11" width="9.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.83203125" style="1"/>
     <col min="13" max="13" width="55" style="17" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="60.6640625" style="2" bestFit="1" customWidth="1"/>
-    <col min="15" max="16384" width="8.88671875" style="2"/>
+    <col min="15" max="16384" width="8.83203125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C1" s="6"/>
       <c r="M1" s="2"/>
     </row>
-    <row r="2" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="9" t="s">
         <v>0</v>
       </c>
@@ -1391,10 +1439,10 @@
         <v>14</v>
       </c>
       <c r="N2" s="11" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="15">
         <f>IF(B3&lt;&gt;"",COUNTA($B$3:B3),"")</f>
         <v>1</v>
@@ -1427,12 +1475,12 @@
         <v>33</v>
       </c>
       <c r="L3" s="22" t="s">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="M3" s="16"/>
       <c r="N3" s="16"/>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="15">
         <f>IF(B4&lt;&gt;"",COUNTA($B$3:B4),"")</f>
         <v>2</v>
@@ -1447,7 +1495,7 @@
         <v>29</v>
       </c>
       <c r="E4" s="15">
-        <v>43.2</v>
+        <v>46</v>
       </c>
       <c r="F4" s="15">
         <v>0</v>
@@ -1463,29 +1511,29 @@
       </c>
       <c r="J4" s="15">
         <f>(G4*E4)+F4</f>
-        <v>43.2</v>
+        <v>46</v>
       </c>
       <c r="K4" s="15" t="s">
         <v>44</v>
       </c>
       <c r="L4" s="22" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="M4" s="16" t="s">
         <v>46</v>
       </c>
       <c r="N4" s="16"/>
     </row>
-    <row r="5" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="15">
         <f>IF(B5&lt;&gt;"",COUNTA($B$3:B5),"")</f>
         <v>3</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D5" s="15" t="s">
         <v>24</v>
@@ -1500,27 +1548,27 @@
         <v>1</v>
       </c>
       <c r="H5" s="15" t="s">
+        <v>112</v>
+      </c>
+      <c r="I5" s="8" t="s">
         <v>113</v>
-      </c>
-      <c r="I5" s="8" t="s">
-        <v>114</v>
       </c>
       <c r="J5" s="15">
         <f>(G5*E5)+F5</f>
         <v>17.96</v>
       </c>
       <c r="K5" s="15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="L5" s="22" t="s">
         <v>12</v>
       </c>
       <c r="M5" s="18" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="N5" s="16"/>
     </row>
-    <row r="6" spans="1:14" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" ht="48" x14ac:dyDescent="0.2">
       <c r="A6" s="15">
         <f>IF(B6&lt;&gt;"",COUNTA($B$3:B6),"")</f>
         <v>4</v>
@@ -1529,7 +1577,7 @@
         <v>40</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D6" s="15" t="s">
         <v>24</v>
@@ -1544,27 +1592,27 @@
         <v>1</v>
       </c>
       <c r="H6" s="15" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="I6" s="8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="J6" s="15">
         <f>(G6*E6)+F6</f>
         <v>33.32</v>
       </c>
       <c r="K6" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L6" s="22" t="s">
         <v>12</v>
       </c>
       <c r="M6" s="18" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="N6" s="16"/>
     </row>
-    <row r="7" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="15">
         <f>IF(B7&lt;&gt;"",COUNTA($B$3:B7),"")</f>
         <v>5</v>
@@ -1591,24 +1639,24 @@
         <v>4</v>
       </c>
       <c r="I7" s="8" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J7" s="15">
         <f t="shared" ref="J7:J23" si="0">(G7*E7)+F7</f>
         <v>143.63</v>
       </c>
       <c r="K7" s="23" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L7" s="22" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M7" s="18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="N7" s="16"/>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="15">
         <f>IF(B8&lt;&gt;"",COUNTA($B$3:B8),"")</f>
         <v>6</v>
@@ -1633,24 +1681,24 @@
         <v>4</v>
       </c>
       <c r="I8" s="8" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J8" s="15">
         <f t="shared" si="0"/>
         <v>25.66</v>
       </c>
       <c r="K8" s="23" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L8" s="22" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M8" s="16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="N8" s="16"/>
     </row>
-    <row r="9" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="15">
         <f>IF(B9&lt;&gt;"",COUNTA($B$3:B9),"")</f>
         <v>7</v>
@@ -1677,7 +1725,7 @@
         <v>4</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="J9" s="15">
         <f t="shared" si="0"/>
@@ -1690,11 +1738,11 @@
         <v>12</v>
       </c>
       <c r="M9" s="18" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="N9" s="27"/>
     </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A10" s="15">
         <f>IF(B10&lt;&gt;"",COUNTA($B$3:B10),"")</f>
         <v>8</v>
@@ -1722,18 +1770,20 @@
         <v>0</v>
       </c>
       <c r="L10" s="22" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="M10" s="16"/>
-      <c r="N10" s="16"/>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="N10" s="16" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A11" s="15">
         <f>IF(B11&lt;&gt;"",COUNTA($B$3:B11),"")</f>
         <v>9</v>
       </c>
       <c r="B11" s="28" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11" s="13" t="s">
         <v>51</v>
@@ -1754,32 +1804,32 @@
         <v>4</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J11" s="15">
         <f t="shared" si="0"/>
         <v>243</v>
       </c>
       <c r="K11" s="15" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="L11" s="22" t="s">
         <v>13</v>
       </c>
       <c r="M11" s="16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="N11" s="16" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A12" s="15">
         <f>IF(B12&lt;&gt;"",COUNTA($B$3:B12),"")</f>
         <v>10</v>
       </c>
       <c r="B12" s="24" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C12" s="13" t="s">
         <v>51</v>
@@ -1800,30 +1850,30 @@
         <v>4</v>
       </c>
       <c r="I12" s="31" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="J12" s="15">
         <f t="shared" si="0"/>
         <v>208.57</v>
       </c>
       <c r="K12" s="23" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="L12" s="22" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="M12" s="16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="N12" s="16"/>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A13" s="15">
         <f>IF(B13&lt;&gt;"",COUNTA($B$3:B13),"")</f>
         <v>11</v>
       </c>
       <c r="B13" s="24" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C13" s="13" t="s">
         <v>51</v>
@@ -1844,35 +1894,35 @@
         <v>4</v>
       </c>
       <c r="I13" s="8" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="J13" s="15">
         <f t="shared" si="0"/>
         <v>150.07</v>
       </c>
       <c r="K13" s="23" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="L13" s="22" t="s">
         <v>13</v>
       </c>
       <c r="M13" s="16" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="N13" s="16" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A14" s="15">
         <f>IF(B14&lt;&gt;"",COUNTA($B$3:B14),"")</f>
         <v>12</v>
       </c>
       <c r="B14" s="24" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D14" s="15" t="s">
         <v>18</v>
@@ -1890,7 +1940,7 @@
         <v>4</v>
       </c>
       <c r="I14" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J14" s="15">
         <f t="shared" si="0"/>
@@ -1900,20 +1950,20 @@
         <v>48</v>
       </c>
       <c r="L14" s="22" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M14" s="16" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="N14" s="16"/>
     </row>
-    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A15" s="15">
         <f>IF(B15&lt;&gt;"",COUNTA($B$3:B15),"")</f>
         <v>13</v>
       </c>
       <c r="B15" s="28" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C15" s="13" t="s">
         <v>52</v>
@@ -1941,16 +1991,16 @@
       <c r="M15" s="16"/>
       <c r="N15" s="16"/>
     </row>
-    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="15">
         <f>IF(B16&lt;&gt;"",COUNTA($B$3:B16),"")</f>
         <v>14</v>
       </c>
       <c r="B16" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="C16" s="13" t="s">
         <v>57</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>58</v>
       </c>
       <c r="D16" s="15" t="s">
         <v>25</v>
@@ -1975,7 +2025,7 @@
       <c r="M16" s="16"/>
       <c r="N16" s="16"/>
     </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="15">
         <f>IF(B17&lt;&gt;"",COUNTA($B$3:B17),"")</f>
         <v>15</v>
@@ -1984,7 +2034,7 @@
         <v>53</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D17" s="15" t="s">
         <v>18</v>
@@ -2002,33 +2052,33 @@
         <v>4</v>
       </c>
       <c r="I17" s="8" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="J17" s="15">
         <f t="shared" si="0"/>
         <v>222.3</v>
       </c>
       <c r="K17" s="15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="L17" s="22" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M17" s="16" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="N17" s="16"/>
     </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A18" s="15">
         <f>IF(B18&lt;&gt;"",COUNTA($B$3:B18),"")</f>
         <v>16</v>
       </c>
       <c r="B18" s="13" t="s">
+        <v>65</v>
+      </c>
+      <c r="C18" s="13" t="s">
         <v>66</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>67</v>
       </c>
       <c r="D18" s="15" t="s">
         <v>25</v>
@@ -2046,33 +2096,33 @@
         <v>4</v>
       </c>
       <c r="I18" s="8" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J18" s="15">
         <f t="shared" si="0"/>
         <v>63.99</v>
       </c>
       <c r="K18" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L18" s="22" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M18" s="16" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="N18" s="16"/>
     </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A19" s="15">
         <f>IF(B19&lt;&gt;"",COUNTA($B$3:B19),"")</f>
         <v>17</v>
       </c>
-      <c r="B19" s="24" t="s">
-        <v>54</v>
+      <c r="B19" s="14" t="s">
+        <v>163</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D19" s="15" t="s">
         <v>25</v>
@@ -2085,28 +2135,31 @@
       <c r="H19" s="15" t="s">
         <v>4</v>
       </c>
-      <c r="I19" s="3"/>
+      <c r="I19" s="3" t="s">
+        <v>164</v>
+      </c>
       <c r="J19" s="15">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="K19" s="15"/>
+        <v>37.6</v>
+      </c>
+      <c r="K19" s="15" t="s">
+        <v>133</v>
+      </c>
       <c r="L19" s="22" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="M19" s="16"/>
       <c r="N19" s="16"/>
     </row>
-    <row r="20" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:14" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" s="15">
         <f>IF(B20&lt;&gt;"",COUNTA($B$3:B20),"")</f>
         <v>18</v>
       </c>
       <c r="B20" s="24" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>30</v>
@@ -2124,33 +2177,33 @@
         <v>4</v>
       </c>
       <c r="I20" s="8" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="J20" s="15">
         <f t="shared" si="0"/>
         <v>17.79</v>
       </c>
       <c r="K20" s="15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="L20" s="22" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M20" s="16" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="N20" s="16"/>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A21" s="15">
         <f>IF(B21&lt;&gt;"",COUNTA($B$3:B21),"")</f>
         <v>19</v>
       </c>
       <c r="B21" s="24" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D21" s="15" t="s">
         <v>30</v>
@@ -2168,7 +2221,7 @@
         <v>4</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="J21" s="15">
         <f t="shared" si="0"/>
@@ -2181,20 +2234,20 @@
         <v>36</v>
       </c>
       <c r="M21" s="16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="N21" s="16"/>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="15">
         <f>IF(B22&lt;&gt;"",COUNTA($B$3:B22),"")</f>
         <v>20</v>
       </c>
       <c r="B22" s="24" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D22" s="15" t="s">
         <v>30</v>
@@ -2212,7 +2265,7 @@
         <v>4</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="J22" s="15">
         <f t="shared" si="0"/>
@@ -2225,20 +2278,20 @@
         <v>36</v>
       </c>
       <c r="M22" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N22" s="16"/>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A23" s="15">
         <f>IF(B23&lt;&gt;"",COUNTA($B$3:B23),"")</f>
         <v>21</v>
       </c>
       <c r="B23" s="24" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D23" s="15" t="s">
         <v>30</v>
@@ -2256,7 +2309,7 @@
         <v>4</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J23" s="15">
         <f t="shared" si="0"/>
@@ -2269,20 +2322,20 @@
         <v>36</v>
       </c>
       <c r="M23" s="16" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="N23" s="16"/>
     </row>
-    <row r="24" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:14" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="15">
         <f>IF(B24&lt;&gt;"",COUNTA($B$3:B24),"")</f>
         <v>22</v>
       </c>
       <c r="B24" s="26" t="s">
+        <v>77</v>
+      </c>
+      <c r="C24" s="13" t="s">
         <v>78</v>
-      </c>
-      <c r="C24" s="13" t="s">
-        <v>79</v>
       </c>
       <c r="D24" s="15" t="s">
         <v>30</v>
@@ -2300,7 +2353,7 @@
         <v>4</v>
       </c>
       <c r="I24" s="13" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="J24" s="15">
         <f t="shared" ref="J24:J30" si="1">(G24*E24)+F24</f>
@@ -2315,16 +2368,16 @@
       <c r="M24" s="16"/>
       <c r="N24" s="16"/>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="15">
         <f>IF(B25&lt;&gt;"",COUNTA($B$3:B25),"")</f>
         <v>23</v>
       </c>
       <c r="B25" s="24" t="s">
+        <v>145</v>
+      </c>
+      <c r="C25" s="13" t="s">
         <v>147</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>149</v>
       </c>
       <c r="D25" s="15" t="s">
         <v>25</v>
@@ -2342,33 +2395,33 @@
         <v>4</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="J25" s="15">
         <f t="shared" si="1"/>
         <v>175.97</v>
       </c>
       <c r="K25" s="15" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="L25" s="22" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M25" s="16" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="N25" s="16"/>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A26" s="15">
         <f>IF(B26&lt;&gt;"",COUNTA($B$3:B26),"")</f>
         <v>24</v>
       </c>
       <c r="B26" s="24" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D26" s="15" t="s">
         <v>25</v>
@@ -2386,33 +2439,35 @@
         <v>4</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="J26" s="15">
         <f t="shared" si="1"/>
         <v>698.08999999999992</v>
       </c>
       <c r="K26" s="15" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="L26" s="22" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="M26" s="16" t="s">
-        <v>150</v>
-      </c>
-      <c r="N26" s="16"/>
-    </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.3">
+        <v>148</v>
+      </c>
+      <c r="N26" s="16" t="s">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A27" s="15">
         <f>IF(B27&lt;&gt;"",COUNTA($B$3:B27),"")</f>
         <v>25</v>
       </c>
       <c r="B27" s="13" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C27" s="13" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D27" s="15" t="s">
         <v>18</v>
@@ -2430,33 +2485,33 @@
         <v>4</v>
       </c>
       <c r="I27" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J27" s="15">
         <f t="shared" si="1"/>
         <v>174.99</v>
       </c>
       <c r="K27" s="15" t="s">
+        <v>86</v>
+      </c>
+      <c r="L27" s="22" t="s">
+        <v>11</v>
+      </c>
+      <c r="M27" s="16" t="s">
         <v>87</v>
       </c>
-      <c r="L27" s="22" t="s">
-        <v>10</v>
-      </c>
-      <c r="M27" s="16" t="s">
-        <v>88</v>
-      </c>
       <c r="N27" s="16"/>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A28" s="15">
         <f>IF(B28&lt;&gt;"",COUNTA($B$3:B28),"")</f>
         <v>26</v>
       </c>
       <c r="B28" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="C28" s="13" t="s">
         <v>63</v>
-      </c>
-      <c r="C28" s="13" t="s">
-        <v>64</v>
       </c>
       <c r="D28" s="15" t="s">
         <v>19</v>
@@ -2474,33 +2529,33 @@
         <v>4</v>
       </c>
       <c r="I28" s="8" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="J28" s="15">
         <f t="shared" si="1"/>
         <v>40.369999999999997</v>
       </c>
       <c r="K28" s="15" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="L28" s="22" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M28" s="16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="N28" s="16"/>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A29" s="15">
         <f>IF(B29&lt;&gt;"",COUNTA($B$3:B29),"")</f>
         <v>27</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>144</v>
+        <v>168</v>
       </c>
       <c r="D29" s="15" t="s">
         <v>28</v>
@@ -2518,33 +2573,35 @@
         <v>4</v>
       </c>
       <c r="I29" s="8" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="J29" s="15">
         <f t="shared" si="1"/>
         <v>53.49</v>
       </c>
       <c r="K29" s="15" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="L29" s="22" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="M29" s="16" t="s">
-        <v>140</v>
-      </c>
-      <c r="N29" s="16"/>
-    </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.3">
+        <v>139</v>
+      </c>
+      <c r="N29" s="16" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A30" s="15">
         <f>IF(B30&lt;&gt;"",COUNTA($B$3:B30),"")</f>
         <v>28</v>
       </c>
       <c r="B30" s="13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C30" s="13" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D30" s="15" t="s">
         <v>25</v>
@@ -2569,16 +2626,16 @@
       <c r="M30" s="16"/>
       <c r="N30" s="16"/>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A31" s="15">
         <f>IF(B31&lt;&gt;"",COUNTA($B$3:B31),"")</f>
         <v>29</v>
       </c>
       <c r="B31" s="19" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C31" s="19" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D31" s="15" t="s">
         <v>25</v>
@@ -2594,29 +2651,31 @@
         <v>4</v>
       </c>
       <c r="I31" s="20" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="J31" s="15">
         <f t="shared" ref="J31" si="2">(G31*E31)+F31</f>
         <v>27.96</v>
       </c>
-      <c r="K31" s="15"/>
+      <c r="K31" s="15" t="s">
+        <v>133</v>
+      </c>
       <c r="L31" s="22" t="s">
-        <v>36</v>
+        <v>11</v>
       </c>
       <c r="M31" s="16"/>
       <c r="N31" s="16"/>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A32" s="15">
         <f>IF(B32&lt;&gt;"",COUNTA($B$3:B32),"")</f>
         <v>30</v>
       </c>
       <c r="B32" s="19" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C32" s="19" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D32" s="15" t="s">
         <v>25</v>
@@ -2632,7 +2691,7 @@
         <v>4</v>
       </c>
       <c r="I32" s="20" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J32" s="15">
         <f t="shared" ref="J32" si="3">(G32*E32)+F32</f>
@@ -2644,19 +2703,19 @@
       </c>
       <c r="M32" s="16"/>
       <c r="N32" s="16" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="33" spans="1:14" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A33" s="15">
         <f>IF(B33&lt;&gt;"",COUNTA($B$3:B33),"")</f>
         <v>31</v>
       </c>
       <c r="B33" s="19" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C33" s="19" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D33" s="15" t="s">
         <v>25</v>
@@ -2672,7 +2731,7 @@
         <v>4</v>
       </c>
       <c r="I33" s="20" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="J33" s="15">
         <f t="shared" ref="J33" si="4">(G33*E33)+F33</f>
@@ -2684,19 +2743,19 @@
       </c>
       <c r="M33" s="16"/>
       <c r="N33" s="16" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="34" spans="1:14" x14ac:dyDescent="0.3">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" ht="16" x14ac:dyDescent="0.2">
       <c r="A34" s="15">
         <f>IF(B34&lt;&gt;"",COUNTA($B$3:B34),"")</f>
         <v>32</v>
       </c>
       <c r="B34" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="C34" s="19" t="s">
         <v>105</v>
-      </c>
-      <c r="C34" s="19" t="s">
-        <v>106</v>
       </c>
       <c r="D34" s="15" t="s">
         <v>25</v>
@@ -2712,47 +2771,154 @@
         <v>4</v>
       </c>
       <c r="I34" s="20" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="J34" s="15">
         <f t="shared" ref="J34" si="5">(G34*E34)+F34</f>
         <v>4.8899999999999997</v>
       </c>
-      <c r="K34" s="15"/>
+      <c r="K34" s="15" t="s">
+        <v>133</v>
+      </c>
       <c r="L34" s="22" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="M34" s="16"/>
       <c r="N34" s="16"/>
     </row>
-    <row r="35" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A35" s="15" t="str">
-        <f>IF(B35&lt;&gt;"",COUNTA($B$3:B35),"")</f>
-        <v/>
-      </c>
-      <c r="L35" s="22"/>
-    </row>
-    <row r="36" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A36" s="15" t="str">
-        <f>IF(B36&lt;&gt;"",COUNTA($B$3:B36),"")</f>
-        <v/>
-      </c>
-      <c r="L36" s="22"/>
-    </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="L37" s="22"/>
-    </row>
-    <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="L38" s="22"/>
-    </row>
-    <row r="39" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="L39" s="22"/>
-    </row>
-    <row r="40" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="L40" s="22"/>
-    </row>
-    <row r="41" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="L41" s="22"/>
+    <row r="35" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+      <c r="A35" s="15">
+        <v>33</v>
+      </c>
+      <c r="B35" s="19" t="s">
+        <v>153</v>
+      </c>
+      <c r="C35" s="19" t="s">
+        <v>170</v>
+      </c>
+      <c r="D35" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15">
+        <v>1</v>
+      </c>
+      <c r="H35" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I35" s="20" t="s">
+        <v>157</v>
+      </c>
+      <c r="J35" s="15">
+        <v>242.17</v>
+      </c>
+      <c r="K35" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="L35" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M35" s="19" t="s">
+        <v>156</v>
+      </c>
+      <c r="N35" s="16"/>
+    </row>
+    <row r="36" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+      <c r="A36" s="15">
+        <v>34</v>
+      </c>
+      <c r="B36" s="19" t="s">
+        <v>159</v>
+      </c>
+      <c r="C36" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D36" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15">
+        <v>1</v>
+      </c>
+      <c r="H36" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I36" s="20" t="s">
+        <v>161</v>
+      </c>
+      <c r="J36" s="15">
+        <v>28.38</v>
+      </c>
+      <c r="K36" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="L36" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M36" s="19" t="s">
+        <v>160</v>
+      </c>
+      <c r="N36" s="16"/>
+    </row>
+    <row r="37" spans="1:14" ht="16" x14ac:dyDescent="0.2">
+      <c r="A37" s="15">
+        <v>35</v>
+      </c>
+      <c r="B37" s="19" t="s">
+        <v>154</v>
+      </c>
+      <c r="C37" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="D37" s="15" t="s">
+        <v>19</v>
+      </c>
+      <c r="E37" s="15"/>
+      <c r="F37" s="15"/>
+      <c r="G37" s="15">
+        <v>1</v>
+      </c>
+      <c r="H37" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="I37" s="20" t="s">
+        <v>158</v>
+      </c>
+      <c r="J37" s="15">
+        <v>264.17</v>
+      </c>
+      <c r="K37" s="15" t="s">
+        <v>162</v>
+      </c>
+      <c r="L37" s="22" t="s">
+        <v>36</v>
+      </c>
+      <c r="M37" s="19" t="s">
+        <v>155</v>
+      </c>
+      <c r="N37" s="16"/>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="K38" s="2"/>
+      <c r="L38" s="2"/>
+      <c r="M38" s="2"/>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="K39" s="2"/>
+      <c r="L39" s="2"/>
+      <c r="M39" s="2"/>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="K40" s="2"/>
+      <c r="L40" s="2"/>
+      <c r="M40" s="2"/>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.2">
+      <c r="K41" s="2"/>
+      <c r="L41" s="2"/>
+      <c r="M41" s="2"/>
     </row>
   </sheetData>
   <autoFilter ref="A2:N34" xr:uid="{0E734346-BCBC-4D9C-B399-F93315446069}"/>
@@ -2760,7 +2926,7 @@
     <mergeCell ref="F7:F8"/>
   </mergeCells>
   <phoneticPr fontId="6" type="noConversion"/>
-  <conditionalFormatting sqref="L3:L6 L10:L12 L15:L26 L28:L41">
+  <conditionalFormatting sqref="L3:L6 L10:L12 L15:L26 L28:L37">
     <cfRule type="containsText" dxfId="7" priority="1" operator="containsText" text="pending">
       <formula>NOT(ISERROR(SEARCH("pending",L3)))</formula>
     </cfRule>
@@ -2768,7 +2934,7 @@
       <formula>$B2="approved"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L3:L41">
+  <conditionalFormatting sqref="L3:L37">
     <cfRule type="containsText" dxfId="6" priority="3" operator="containsText" text="approved">
       <formula>NOT(ISERROR(SEARCH("approved",L3)))</formula>
     </cfRule>
@@ -2782,7 +2948,7 @@
       <formula>NOT(ISERROR(SEARCH("received",L3)))</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L4:L41">
+  <conditionalFormatting sqref="L4:L37">
     <cfRule type="expression" priority="9">
       <formula>#REF!="approved"</formula>
     </cfRule>
@@ -2849,19 +3015,19 @@
           <x14:formula1>
             <xm:f>Background_info!$D$3:$D$30</xm:f>
           </x14:formula1>
-          <xm:sqref>D3:D34</xm:sqref>
+          <xm:sqref>D3:D37</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{0CED9412-699B-4C7D-965B-005ACFAE9885}">
           <x14:formula1>
             <xm:f>Background_info!$C$3:$C$15</xm:f>
           </x14:formula1>
-          <xm:sqref>L3:L41</xm:sqref>
+          <xm:sqref>L3:L37</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4580CAC9-FAF7-403B-A1D9-84CB43CB97A9}">
           <x14:formula1>
             <xm:f>Background_info!$B$3:$B$7</xm:f>
           </x14:formula1>
-          <xm:sqref>H3:H34</xm:sqref>
+          <xm:sqref>H3:H37</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2872,13 +3038,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2F602BA-A80C-4BEA-8ECF-F81C395286C3}">
   <dimension ref="A1:G14"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="33" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B1" t="str" cm="1">
         <f t="array" ref="B1:F1">TRANSPOSE(Background_info!C3:C7)</f>
         <v>pending</v>
@@ -2896,36 +3062,36 @@
         <v>rejected</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B2" s="30">
         <f>SUM(B3:B14)</f>
-        <v>763.17</v>
+        <v>780.41</v>
       </c>
       <c r="C2" s="30">
         <f t="shared" ref="C2:F2" si="0">SUM(C3:C14)</f>
-        <v>1207.75</v>
+        <v>0</v>
       </c>
       <c r="D2" s="30">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>968.05</v>
       </c>
       <c r="E2" s="30">
         <f t="shared" si="0"/>
-        <v>120.78</v>
+        <v>166.78</v>
       </c>
       <c r="F2" s="30">
         <f t="shared" si="0"/>
-        <v>421.83</v>
+        <v>1173.4099999999999</v>
       </c>
       <c r="G2" s="29">
         <f>SUM(B2:F2)</f>
-        <v>2513.5300000000002</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+        <v>3088.6499999999996</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" t="str" cm="1">
         <f t="array" ref="A3:A14">Background_info!D3:D14</f>
         <v>Airframe and Structures</v>
@@ -2936,11 +3102,11 @@
       </c>
       <c r="C3">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A3,Main_Table!$L:$L,C$1)</f>
-        <v>169.29</v>
+        <v>0</v>
       </c>
       <c r="D3">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A3,Main_Table!$L:$L,D$1)</f>
-        <v>0</v>
+        <v>169.29</v>
       </c>
       <c r="E3">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A3,Main_Table!$L:$L,E$1)</f>
@@ -2951,7 +3117,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="str">
         <v>Propulsion</v>
       </c>
@@ -2961,11 +3127,11 @@
       </c>
       <c r="C4">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A4,Main_Table!$L:$L,C$1)</f>
-        <v>430.19000000000005</v>
+        <v>0</v>
       </c>
       <c r="D4">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A4,Main_Table!$L:$L,D$1)</f>
-        <v>0</v>
+        <v>430.19000000000005</v>
       </c>
       <c r="E4">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A4,Main_Table!$L:$L,E$1)</f>
@@ -2976,21 +3142,21 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="str">
         <v>Power</v>
       </c>
       <c r="B5">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A5,Main_Table!$L:$L,B$1)</f>
-        <v>0</v>
+        <v>472.74</v>
       </c>
       <c r="C5">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A5,Main_Table!$L:$L,C$1)</f>
-        <v>248.94</v>
+        <v>0</v>
       </c>
       <c r="D5">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A5,Main_Table!$L:$L,D$1)</f>
-        <v>0</v>
+        <v>40.369999999999997</v>
       </c>
       <c r="E5">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A5,Main_Table!$L:$L,E$1)</f>
@@ -3001,21 +3167,21 @@
         <v>393.07</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" t="str">
         <v>Flight Control and Avionics</v>
       </c>
       <c r="B6">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A6,Main_Table!$L:$L,B$1)</f>
-        <v>726.05</v>
+        <v>0</v>
       </c>
       <c r="C6">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A6,Main_Table!$L:$L,C$1)</f>
-        <v>244.85</v>
+        <v>0</v>
       </c>
       <c r="D6">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A6,Main_Table!$L:$L,D$1)</f>
-        <v>0</v>
+        <v>310.40999999999997</v>
       </c>
       <c r="E6">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A6,Main_Table!$L:$L,E$1)</f>
@@ -3023,10 +3189,10 @@
       </c>
       <c r="F6">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A6,Main_Table!$L:$L,F$1)</f>
-        <v>28.76</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>726.84999999999991</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" t="str">
         <v>Control Surfaces and Mechanisms</v>
       </c>
@@ -3051,7 +3217,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" t="str">
         <v>Payload and Medical Transport System</v>
       </c>
@@ -3076,17 +3242,17 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" t="str">
         <v>Communications and Ground Equipment</v>
       </c>
       <c r="B9">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A9,Main_Table!$L:$L,B$1)</f>
-        <v>0</v>
+        <v>270.55</v>
       </c>
       <c r="C9">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A9,Main_Table!$L:$L,C$1)</f>
-        <v>53.49</v>
+        <v>0</v>
       </c>
       <c r="D9">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A9,Main_Table!$L:$L,D$1)</f>
@@ -3098,10 +3264,10 @@
       </c>
       <c r="F9">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A9,Main_Table!$L:$L,F$1)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <v>53.49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A10" t="str">
         <v>Manufacturing and prototyping</v>
       </c>
@@ -3111,7 +3277,7 @@
       </c>
       <c r="C10">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A10,Main_Table!$L:$L,C$1)</f>
-        <v>43.2</v>
+        <v>0</v>
       </c>
       <c r="D10">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A10,Main_Table!$L:$L,D$1)</f>
@@ -3119,14 +3285,14 @@
       </c>
       <c r="E10">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A10,Main_Table!$L:$L,E$1)</f>
-        <v>69.5</v>
+        <v>115.5</v>
       </c>
       <c r="F10">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A10,Main_Table!$L:$L,F$1)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" t="str">
         <v>Fasteners and Consumables</v>
       </c>
@@ -3136,11 +3302,11 @@
       </c>
       <c r="C11">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A11,Main_Table!$L:$L,C$1)</f>
-        <v>17.79</v>
+        <v>0</v>
       </c>
       <c r="D11">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A11,Main_Table!$L:$L,D$1)</f>
-        <v>0</v>
+        <v>17.79</v>
       </c>
       <c r="E11">
         <f>SUMIFS(Main_Table!$J:$J,Main_Table!$D:$D,$A11,Main_Table!$L:$L,E$1)</f>
@@ -3151,7 +3317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" t="str">
         <v>Testing and Safety Equipment</v>
       </c>
@@ -3176,7 +3342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" t="str">
         <v>Business</v>
       </c>
@@ -3201,7 +3367,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" t="str">
         <v>Other</v>
       </c>

</xml_diff>